<commit_message>
Add leaveGuard functionality with tests for sheet closing behavior
- Implement leaveGuard.ts to manage sheet closing scenarios, including cloud and file states.
- Create leaveGuard.test.ts to validate the behavior of leave reasons, messages, and save actions.
- Update fontSizes.test.ts to explicitly type variable for clarity.
</commit_message>
<xml_diff>
--- a/Cowork changes 4 Sep 2026.xlsx
+++ b/Cowork changes 4 Sep 2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="572">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="652">
   <si>
     <t>Cowork — changes, 4 September 2026</t>
   </si>
@@ -959,6 +959,27 @@
     <t>5 September 2026</t>
   </si>
   <si>
+    <t>1k</t>
+  </si>
+  <si>
+    <t>Task chat ▸ Add submission</t>
+  </si>
+  <si>
+    <t>The submission dialog is opaque</t>
+  </si>
+  <si>
+    <t>The task page read straight through it. The dialog paints no surface of its own by design — the form inside brings its own panel — but that panel is 74% transparent and hides what is behind it with a backdrop blur, which holds over the page's own quiet ground and fails over a busy one. The form and the thread's cards were drawn over each other, both legible, neither readable.</t>
+  </si>
+  <si>
+    <t>A solid panel colour, and a heavier scrim. Measured in a browser: a plain frosted panel computes rgba(32,32,37,0.74); inside the dialog it computes rgb(32,32,37).</t>
+  </si>
+  <si>
+    <t>The original reasoning — that a modal needs no surface because its child has one — was wrong about WHICH surface. A translucent panel is a surface for the page it belongs to, not for an arbitrary one behind a portal. Done by overriding the colour token rather than laying an opaque div under the child: the property inherits, so there is no second element whose corners and border have to be kept in step with the panel's own.</t>
+  </si>
+  <si>
+    <t>app/globals.css (--frost-panel-solid); components/features/tasks/TaskChatSubmission.tsx (+ submitDialog test)</t>
+  </si>
+  <si>
     <t>3c</t>
   </si>
   <si>
@@ -1034,6 +1055,66 @@
     <t>app/globals.css; components/features/spreadsheet/Spreadsheet.tsx (+ chromeSelection test)</t>
   </si>
   <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>The Overview dashboard</t>
+  </si>
+  <si>
+    <t>Requested: the Needs you panel should reach the bottom of the page rather than stopping short of the left-hand column.</t>
+  </si>
+  <si>
+    <t>8a</t>
+  </si>
+  <si>
+    <t>Overview ▸ Needs you</t>
+  </si>
+  <si>
+    <t>The panel fills its column</t>
+  </si>
+  <si>
+    <t>It packed to its rows, so the right-hand column stopped well above the left one and the page ended on a ragged edge.</t>
+  </si>
+  <si>
+    <t>It holds the rest of the column, so the two regions end on one line. Measured before and after in a browser: the card went from ending at 301px to filling its wrapper exactly at 471px.</t>
+  </si>
+  <si>
+    <t>**This reverses a documented decision, and a test that guarded it.** The card was deliberately shortened because the list is capped at six rows, and empty card below its own content was judged to read as a loading failure. The counter-argument that won: a right column stopping short reads as unfinished at EVERY window size and does so all the time, whereas the empty band only shows when there are few signals. If it becomes a nuisance the fix is to let the list use the extra height — raise the cap and scroll — rather than to shorten the card again.</t>
+  </si>
+  <si>
+    <t>components/features/dashboard/Home.tsx; AttentionCard.tsx; signals.test.ts (guard reversed, with the decision recorded in it)</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>The brief card in a task chat</t>
+  </si>
+  <si>
+    <t>Requested: move Open the task to the top right of the card and make it the product's white button.</t>
+  </si>
+  <si>
+    <t>9a</t>
+  </si>
+  <si>
+    <t>Task chat ▸ the brief card, expanded</t>
+  </si>
+  <si>
+    <t>Open the task moved to the top right, as the primary button</t>
+  </si>
+  <si>
+    <t>A quiet grey text link at the FOOT of the panel, under the deliverables — so on a task with a long brief it sat below the fold of the card, and the only control in there was the last thing anybody found.</t>
+  </si>
+  <si>
+    <t>A white pill on the first line, beside the brief, where the eye already is. It does not move when the brief grows.</t>
+  </si>
+  <si>
+    <t>'Our white button' is `bg-ink` on `--body-bg` ink — so it reads white on dark and dark on light without either colour being written into this card. Sized to the card's 11px type rather than the standard 13px: a full-height button in a panel of small print reads as something pasted in. Verified in a browser — the pill sits 10px from the panel's top and 12px from its right, on rgb(241,241,243) with dark ink and a full radius.</t>
+  </si>
+  <si>
+    <t>components/features/messages/TaskChatBrief.tsx</t>
+  </si>
+  <si>
     <t>What is open</t>
   </si>
   <si>
@@ -1731,6 +1812,165 @@
   </si>
   <si>
     <t>scratchpad/sheetgen/forktab.js</t>
+  </si>
+  <si>
+    <t>Font size on the spreadsheet ribbon</t>
+  </si>
+  <si>
+    <t>Reported: pressing A+ did not move the number in the box beside it — the two read as unconnected.</t>
+  </si>
+  <si>
+    <t>Sheets ▸ Home ribbon ▸ Font</t>
+  </si>
+  <si>
+    <t>A+ and A− step the size LADDER, not one point</t>
+  </si>
+  <si>
+    <t>The picker offered 10, 11, 12, 13, 14, 16, 18, 24, 32 and the buttons stepped by ONE. Past 14 they disagreed: a press produced 15, which is not on the ladder, so the select had no option matching its own value and stopped showing the size. Press again and it landed on 16 and came back.</t>
+  </si>
+  <si>
+    <t>A press moves one rung — 14 to 16, 16 to 18 — so the number always follows the button. Past the ends it still moves by a point rather than refusing, clamped to 6-96.</t>
+  </si>
+  <si>
+    <t>Reported. The product's own document toolbar already stepped its ladder correctly, in a private helper the spreadsheet could not reach; that logic is now shared and tested rather than copied a third time.</t>
+  </si>
+  <si>
+    <t>lib/spreadsheet/fontSizes.ts (new, 10 tests); HomeTab.tsx</t>
+  </si>
+  <si>
+    <t>Both spreadsheet size pickers</t>
+  </si>
+  <si>
+    <t>A size the ladder does not carry is still shown</t>
+  </si>
+  <si>
+    <t>The list was a fixed nine values, duplicated in the ribbon and the toolbar. Anything else — a size from an opened .xlsx, or one reached before this fix — matched no option and the picker showed nothing.</t>
+  </si>
+  <si>
+    <t>The applied size is added to the options when it is not a rung, and the ladder itself comes from one shared module so the two pickers cannot drift.</t>
+  </si>
+  <si>
+    <t>A control that cannot display its own value is the same defect in a different costume — and opening real files, which the other session has just added, makes off-ladder sizes ordinary rather than rare.</t>
+  </si>
+  <si>
+    <t>lib/spreadsheet/fontSizes.ts; HomeTab.tsx; SpreadsheetToolbar.tsx</t>
+  </si>
+  <si>
+    <t>Putting a sheet down</t>
+  </si>
+  <si>
+    <t>Three requests together: a dropped file should offer Don't save, the browser's back button should ask rather than closing silently, and the File menu should have a Close.</t>
+  </si>
+  <si>
+    <t>Sheets ▸ closing an open sheet</t>
+  </si>
+  <si>
+    <t>Closing asks when something is still unsaved</t>
+  </si>
+  <si>
+    <t>The back arrow shut the sheet on the spot. A sheet autosaves so usually nothing was lost, but 'usually' is not something you can see — and the two unsafe cases, a save still on the wire and a save that FAILED, looked exactly like the safe one.</t>
+  </si>
+  <si>
+    <t>Closing checks both stores and, when either is behind, names which and offers Save / Don't save / Cancel. A clean sheet still closes on the spot; stopping somebody to say nothing was lost is the dialog people learn to dismiss.</t>
+  </si>
+  <si>
+    <t>Requested. Both stores, because a sheet safely in Cowork whose write back to the file on the computer was refused has still lost the copy the person was watching. Save reads 'Try saving again' where the last attempt failed, rather than pretending a retry is a certainty.</t>
+  </si>
+  <si>
+    <t>lib/rules/sheets/leaveGuard.ts (new, 12 tests); Spreadsheet.tsx</t>
+  </si>
+  <si>
+    <t>8b</t>
+  </si>
+  <si>
+    <t>Sheets ▸ the browser's back button</t>
+  </si>
+  <si>
+    <t>Back closes the sheet, and asks first</t>
+  </si>
+  <si>
+    <t>The open sheet is a full-screen layer held in the list's state, not a route — so back left the whole Sheets page, taking the sheet with it and saying nothing about whether the work was stored. `beforeunload` does not fire on a client-side navigation, so nothing caught it.</t>
+  </si>
+  <si>
+    <t>Opening a sheet pushes one history entry and back pops it, so the gesture means 'close this sheet' and goes through the same guard as every other exit.</t>
+  </si>
+  <si>
+    <t>Requested. Cancelling pushes the step BACK — without that the reader spends their one back press to stay where they were, and the next one leaves the page for real.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/Spreadsheet.tsx</t>
+  </si>
+  <si>
+    <t>8c</t>
+  </si>
+  <si>
+    <t>Sheets ▸ File menu</t>
+  </si>
+  <si>
+    <t>A Close item</t>
+  </si>
+  <si>
+    <t>The only way out was the back arrow in the corner. A File menu offering New sheet, Open, Save and Share with no way to put the file down is missing half its own vocabulary.</t>
+  </si>
+  <si>
+    <t>Close, at the foot of the menu under a divider, running the same guarded action as the back arrow. Absent where there is no list to return to.</t>
+  </si>
+  <si>
+    <t>Requested. Last and separated because it is the one item that ends the session with this sheet — a mis-click a pixel below Share should not cost somebody their place.</t>
+  </si>
+  <si>
+    <t>FileMenu.tsx; Ribbon.tsx; Spreadsheet.tsx</t>
+  </si>
+  <si>
+    <t>8d</t>
+  </si>
+  <si>
+    <t>Sheets ▸ dropping a file on an open sheet</t>
+  </si>
+  <si>
+    <t>The drop question gained Don't save</t>
+  </si>
+  <si>
+    <t>Cancel and 'Save and open'. Somebody who did not want to wait for a slow or stuck save had to cancel and lose the drop entirely.</t>
+  </si>
+  <si>
+    <t>Three answers, the same three closing offers.</t>
+  </si>
+  <si>
+    <t>Requested. Don't save does not undo anything — autosave has already stored what it managed — it declines to WAIT for the write still outstanding, and the wording says so rather than the usual 'your changes will be lost', which would be false here.</t>
+  </si>
+  <si>
+    <t>8e</t>
+  </si>
+  <si>
+    <t>The Sheets article covers closing</t>
+  </si>
+  <si>
+    <t>It described the drop question's two answers and said nothing about closing.</t>
+  </si>
+  <si>
+    <t>The three answers, when closing asks and when it does not, what Don't save actually means, that browser back closes the sheet, and where File ▸ Close is.</t>
+  </si>
+  <si>
+    <t>Project rule. The Don't save sentence matters most: a reader who thinks it reverts their work would use it expecting an undo.</t>
+  </si>
+  <si>
+    <t>8f</t>
+  </si>
+  <si>
+    <t>Closing a sheet you CHANGED always confirms</t>
+  </si>
+  <si>
+    <t>8a gated the question on a write being outstanding. Both stores autosave about a second after you stop typing, so a second later everything read `saved` and Close went through in silence — which is exactly what was reported back: make a change, press Close, no prompt. From the outside that is indistinguishable from a sheet that never saved at all.</t>
+  </si>
+  <si>
+    <t>Editing is tracked separately from whether a write is pending, and any sheet that was changed confirms on the way out. Everything stored says so and offers Close / Cancel; something outstanding still offers Save / Don't save / Cancel. A sheet only opened and read still closes straight away.</t>
+  </si>
+  <si>
+    <t>Reported. Don't save is hidden where everything is stored rather than shown doing nothing — autosave cannot be undone, so the button would either be inert or imply a revert, and a choice with no consequence teaches people the whole dialog is decorative. The main button reads Close rather than Save for the same reason.</t>
+  </si>
+  <si>
+    <t>lib/rules/sheets/leaveGuard.ts (+5 tests); Spreadsheet.tsx; lib/help/knowledge.ts</t>
   </si>
 </sst>
 </file>
@@ -2424,7 +2664,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:K56"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -3150,11 +3390,11 @@
         <v>46269.747210648144</v>
       </c>
       <c r="C22" s="8">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D22" s="9">
         <f>C22-B22</f>
-        <v>0.6948842592592592</v>
+        <v>0.7700462962962963</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>167</v>
@@ -3284,11 +3524,11 @@
         <v>46269.773148148146</v>
       </c>
       <c r="C26" s="8">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D26" s="9">
         <f>C26-B26</f>
-        <v>0.6689467592592593</v>
+        <v>0.7441087962962963</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>190</v>
@@ -3454,11 +3694,11 @@
         <v>46269.79305555555</v>
       </c>
       <c r="C31" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D31" s="12">
         <f>C31-B31</f>
-        <v>0.6490393518518518</v>
+        <v>0.7242013888888889</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>219</v>
@@ -3562,11 +3802,11 @@
         <v>46269.82777777778</v>
       </c>
       <c r="C34" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D34" s="12">
         <f>C34-B34</f>
-        <v>0.6143171296296296</v>
+        <v>0.6894791666666666</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>115</v>
@@ -3634,11 +3874,11 @@
         <v>46269.83541666667</v>
       </c>
       <c r="C36" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D36" s="12">
         <f>C36-B36</f>
-        <v>0.6066782407407407</v>
+        <v>0.6818402777777778</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>252</v>
@@ -3768,11 +4008,11 @@
         <v>46269.84722222222</v>
       </c>
       <c r="C40" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D40" s="12">
         <f>C40-B40</f>
-        <v>0.5948726851851852</v>
+        <v>0.6700347222222223</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>273</v>
@@ -3840,11 +4080,11 @@
         <v>46269.813368055555</v>
       </c>
       <c r="C42" s="8">
-        <v>46270.44209490741</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D42" s="9">
         <f>C42-B42</f>
-        <v>0.6287268518518518</v>
+        <v>0.7038888888888889</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>286</v>
@@ -4017,19 +4257,19 @@
       <c r="J47" s="6"/>
       <c r="K47" s="6"/>
     </row>
-    <row r="48" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" ht="146" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
         <v>314</v>
       </c>
       <c r="B48" s="11">
-        <v>46270.42487268518</v>
+        <v>46270.51388888889</v>
       </c>
       <c r="C48" s="11">
-        <v>46270.42679398148</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D48" s="12">
         <f>C48-B48</f>
-        <v>0.0019212962962962964</v>
+        <v>0.0033680555555555556</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>315</v>
@@ -4053,94 +4293,94 @@
         <v>320</v>
       </c>
     </row>
-    <row r="49" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
         <v>321</v>
       </c>
       <c r="B49" s="11">
-        <v>46270.43513888889</v>
+        <v>46270.42487268518</v>
       </c>
       <c r="C49" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.42679398148</v>
       </c>
       <c r="D49" s="12">
         <f>C49-B49</f>
-        <v>0.0069560185185185185</v>
+        <v>0.0019212962962962964</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>161</v>
+        <v>322</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="H49" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="J49" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K49" s="2" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="50" ht="160" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="50" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="10" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B50" s="11">
-        <v>46270.40912037037</v>
+        <v>46270.43513888889</v>
       </c>
       <c r="C50" s="11">
-        <v>46270.42003472222</v>
+        <v>46270.51725694444</v>
       </c>
       <c r="D50" s="12">
         <f>C50-B50</f>
-        <v>0.010914351851851852</v>
+        <v>0.08211805555555556</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>262</v>
+        <v>161</v>
       </c>
       <c r="F50" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K50" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="G50" s="2" t="s">
-        <v>328</v>
-      </c>
-      <c r="H50" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>330</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="K50" s="2" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="51" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" ht="160" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B51" s="11">
-        <v>46270.43833333333</v>
+        <v>46270.40912037037</v>
       </c>
       <c r="C51" s="11">
-        <v>46270.44209490741</v>
+        <v>46270.42003472222</v>
       </c>
       <c r="D51" s="12">
         <f>C51-B51</f>
-        <v>0.003761574074074074</v>
+        <v>0.010914351851851852</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>333</v>
+        <v>262</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>334</v>
@@ -4161,9 +4401,169 @@
         <v>338</v>
       </c>
     </row>
+    <row r="52" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="B52" s="11">
+        <v>46270.43833333333</v>
+      </c>
+      <c r="C52" s="11">
+        <v>46270.51725694444</v>
+      </c>
+      <c r="D52" s="12">
+        <f>C52-B52</f>
+        <v>0.07892361111111111</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B53" s="8">
+        <v>46270.447222222225</v>
+      </c>
+      <c r="C53" s="8">
+        <v>46270.45972222222</v>
+      </c>
+      <c r="D53" s="9">
+        <f>C53-B53</f>
+        <v>0.0125</v>
+      </c>
+      <c r="E53" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="F53" s="7"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="7"/>
+      <c r="I53" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="J53" s="7"/>
+      <c r="K53" s="7"/>
+    </row>
+    <row r="54" ht="188" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="B54" s="11">
+        <v>46270.447222222225</v>
+      </c>
+      <c r="C54" s="11">
+        <v>46270.45972222222</v>
+      </c>
+      <c r="D54" s="12">
+        <f>C54-B54</f>
+        <v>0.0125</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="B55" s="8">
+        <v>46270.461805555555</v>
+      </c>
+      <c r="C55" s="8">
+        <v>46270.46840277778</v>
+      </c>
+      <c r="D55" s="9">
+        <f>C55-B55</f>
+        <v>0.006597222222222222</v>
+      </c>
+      <c r="E55" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F55" s="7"/>
+      <c r="G55" s="7"/>
+      <c r="H55" s="7"/>
+      <c r="I55" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="J55" s="7"/>
+      <c r="K55" s="7"/>
+    </row>
+    <row r="56" ht="146" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="B56" s="11">
+        <v>46270.46388888889</v>
+      </c>
+      <c r="C56" s="11">
+        <v>46270.46840277778</v>
+      </c>
+      <c r="D56" s="12">
+        <f>C56-B56</f>
+        <v>0.0045138888888888885</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K56" s="2" t="s">
+        <v>365</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K51"/>
-  <mergeCells count="9">
+  <autoFilter ref="A1:K56"/>
+  <mergeCells count="11">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="E14:H14"/>
@@ -4173,6 +4573,8 @@
     <mergeCell ref="E37:H37"/>
     <mergeCell ref="E42:H42"/>
     <mergeCell ref="A47:K47"/>
+    <mergeCell ref="E53:H53"/>
+    <mergeCell ref="E55:H55"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4194,13 +4596,13 @@
         <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>339</v>
+        <v>366</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>340</v>
+        <v>367</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>341</v>
+        <v>368</v>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4208,27 +4610,27 @@
         <v>137</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>342</v>
+        <v>369</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>343</v>
+        <v>370</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>344</v>
+        <v>371</v>
       </c>
     </row>
     <row r="3" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>345</v>
+        <v>372</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>346</v>
+        <v>373</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>347</v>
+        <v>374</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>348</v>
+        <v>375</v>
       </c>
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4236,13 +4638,13 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>349</v>
+        <v>376</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>350</v>
+        <v>377</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>351</v>
+        <v>378</v>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4250,13 +4652,13 @@
         <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>352</v>
+        <v>379</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>353</v>
+        <v>380</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>354</v>
+        <v>381</v>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4264,13 +4666,13 @@
         <v>108</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>355</v>
+        <v>382</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>356</v>
+        <v>383</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>357</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4278,13 +4680,13 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>358</v>
+        <v>385</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>359</v>
+        <v>386</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>360</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4292,27 +4694,27 @@
         <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>361</v>
+        <v>388</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>362</v>
+        <v>389</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>363</v>
+        <v>390</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>364</v>
+        <v>391</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>365</v>
+        <v>392</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>366</v>
+        <v>393</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>367</v>
+        <v>394</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4320,13 +4722,13 @@
         <v>251</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>368</v>
+        <v>395</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>369</v>
+        <v>396</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>370</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4334,13 +4736,13 @@
         <v>199</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>371</v>
+        <v>398</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>372</v>
+        <v>399</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>373</v>
+        <v>400</v>
       </c>
     </row>
     <row r="12" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4348,13 +4750,13 @@
         <v>199</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>374</v>
+        <v>401</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>375</v>
+        <v>402</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>376</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4362,27 +4764,27 @@
         <v>199</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>377</v>
+        <v>404</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>378</v>
+        <v>405</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>379</v>
+        <v>406</v>
       </c>
     </row>
     <row r="14" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>380</v>
+        <v>407</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>381</v>
+        <v>408</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>382</v>
+        <v>409</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>383</v>
+        <v>410</v>
       </c>
     </row>
   </sheetData>
@@ -4405,7 +4807,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>384</v>
+        <v>411</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -4418,179 +4820,179 @@
         <v>40</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>385</v>
+        <v>412</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>386</v>
+        <v>413</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>387</v>
+        <v>414</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>388</v>
+        <v>415</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>389</v>
+        <v>416</v>
       </c>
     </row>
     <row r="3" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>390</v>
+        <v>417</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>391</v>
+        <v>418</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>392</v>
+        <v>419</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>393</v>
+        <v>420</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>394</v>
+        <v>421</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="4" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>396</v>
+        <v>423</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>397</v>
+        <v>424</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>398</v>
+        <v>425</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>399</v>
+        <v>426</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>400</v>
+        <v>427</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>401</v>
+        <v>428</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>402</v>
+        <v>429</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>403</v>
+        <v>430</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>404</v>
+        <v>431</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>405</v>
+        <v>432</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>406</v>
+        <v>433</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>407</v>
+        <v>434</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>408</v>
+        <v>435</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>409</v>
+        <v>436</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>410</v>
+        <v>437</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>411</v>
+        <v>438</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8" ht="92" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>412</v>
+        <v>439</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>413</v>
+        <v>440</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>414</v>
+        <v>441</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>415</v>
+        <v>442</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>416</v>
+        <v>443</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>417</v>
+        <v>444</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>418</v>
+        <v>445</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>419</v>
+        <v>446</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>420</v>
+        <v>447</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>395</v>
+        <v>422</v>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>421</v>
+        <v>448</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>449</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>452</v>
+      </c>
+      <c r="F10" s="13" t="s">
         <v>422</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>395</v>
       </c>
     </row>
   </sheetData>
@@ -4604,7 +5006,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K42"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -4703,19 +5105,19 @@
         <v>0.0026504629640839994</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>426</v>
+        <v>453</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -4738,22 +5140,22 @@
         <v>159</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>427</v>
+        <v>454</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>428</v>
+        <v>455</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>429</v>
+        <v>456</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>430</v>
+        <v>457</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>431</v>
+        <v>458</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4771,19 +5173,19 @@
         <v>0.017418981482478557</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>432</v>
+        <v>459</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>432</v>
+        <v>459</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>432</v>
+        <v>459</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>432</v>
+        <v>459</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>433</v>
+        <v>460</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -4803,25 +5205,25 @@
         <v>0.0020370370366435964</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>434</v>
+        <v>461</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>435</v>
+        <v>462</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>436</v>
+        <v>463</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>437</v>
+        <v>464</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>438</v>
+        <v>465</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>439</v>
+        <v>466</v>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4839,25 +5241,25 @@
         <v>0.0026504629640839994</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>440</v>
+        <v>467</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>441</v>
+        <v>468</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>442</v>
+        <v>469</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>443</v>
+        <v>470</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>444</v>
+        <v>471</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>445</v>
+        <v>472</v>
       </c>
     </row>
     <row r="8" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4875,25 +5277,25 @@
         <v>0.00010416666555101983</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>446</v>
+        <v>473</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>447</v>
+        <v>474</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>448</v>
+        <v>475</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>449</v>
+        <v>476</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>450</v>
+        <v>477</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>451</v>
+        <v>478</v>
       </c>
     </row>
     <row r="9" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -4911,30 +5313,30 @@
         <v>0.00028935185036971234</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>452</v>
+        <v>479</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>453</v>
+        <v>480</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>454</v>
+        <v>481</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>455</v>
+        <v>482</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>456</v>
+        <v>483</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>457</v>
+        <v>484</v>
       </c>
     </row>
     <row r="10" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>458</v>
+        <v>485</v>
       </c>
       <c r="B10" s="11">
         <v>46269.77627314815</v>
@@ -4950,27 +5352,27 @@
         <v>115</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>459</v>
+        <v>486</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>460</v>
+        <v>487</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>461</v>
+        <v>488</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>462</v>
+        <v>489</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>463</v>
+        <v>490</v>
       </c>
     </row>
     <row r="11" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>464</v>
+        <v>491</v>
       </c>
       <c r="B11" s="11">
         <v>46269.78513888889</v>
@@ -4983,30 +5385,30 @@
         <v>0.0005555555544560775</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>465</v>
+        <v>492</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>466</v>
+        <v>493</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>467</v>
+        <v>494</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>468</v>
+        <v>495</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>469</v>
+        <v>496</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>457</v>
+        <v>484</v>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>470</v>
+        <v>497</v>
       </c>
       <c r="B12" s="11">
         <v>46269.784733796296</v>
@@ -5019,30 +5421,30 @@
         <v>0.0009606481471564621</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>471</v>
+        <v>498</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>472</v>
+        <v>499</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>473</v>
+        <v>500</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>474</v>
+        <v>501</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>475</v>
+        <v>502</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>476</v>
+        <v>503</v>
       </c>
     </row>
     <row r="13" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>477</v>
+        <v>504</v>
       </c>
       <c r="B13" s="11">
         <v>46269.78622685185</v>
@@ -5058,16 +5460,16 @@
         <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>478</v>
+        <v>505</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>479</v>
+        <v>506</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>480</v>
+        <v>507</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>481</v>
+        <v>508</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>31</v>
@@ -5091,19 +5493,19 @@
         <v>0.0065393518525525</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>483</v>
+        <v>510</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -5123,25 +5525,25 @@
         <v>0.00020833333474001847</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>484</v>
+        <v>511</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>485</v>
+        <v>512</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>486</v>
+        <v>513</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>487</v>
+        <v>514</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>488</v>
+        <v>515</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>489</v>
+        <v>516</v>
       </c>
     </row>
     <row r="16" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5159,30 +5561,30 @@
         <v>0.0016666666670062114</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>490</v>
+        <v>517</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>491</v>
+        <v>518</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>492</v>
+        <v>519</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>494</v>
+        <v>521</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>495</v>
+        <v>522</v>
       </c>
     </row>
     <row r="17" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B17" s="11">
         <v>46269.79986111111</v>
@@ -5198,16 +5600,16 @@
         <v>115</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>496</v>
+        <v>523</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>497</v>
+        <v>524</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>498</v>
+        <v>525</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>499</v>
+        <v>526</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>31</v>
@@ -5231,19 +5633,19 @@
         <v>0.01622685185066075</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>500</v>
+        <v>527</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>500</v>
+        <v>527</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>500</v>
+        <v>527</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>500</v>
+        <v>527</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>501</v>
+        <v>528</v>
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -5263,25 +5665,25 @@
         <v>0.0001851851848186925</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>502</v>
+        <v>529</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>503</v>
+        <v>530</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>504</v>
+        <v>531</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>505</v>
+        <v>532</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>506</v>
+        <v>533</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>507</v>
+        <v>534</v>
       </c>
     </row>
     <row r="20" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5299,25 +5701,25 @@
         <v>0.0015509259246755391</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>508</v>
+        <v>535</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>509</v>
+        <v>536</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>510</v>
+        <v>537</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>511</v>
+        <v>538</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>512</v>
+        <v>539</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>513</v>
+        <v>540</v>
       </c>
     </row>
     <row r="21" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5335,30 +5737,30 @@
         <v>0.001701388890069211</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>514</v>
+        <v>541</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>515</v>
+        <v>542</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>516</v>
+        <v>543</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>518</v>
+        <v>545</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>519</v>
+        <v>546</v>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>520</v>
+        <v>547</v>
       </c>
       <c r="B22" s="11">
         <v>46269.82821759259</v>
@@ -5371,30 +5773,30 @@
         <v>0.0010532407395658083</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>521</v>
+        <v>548</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>522</v>
+        <v>549</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>523</v>
+        <v>550</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>524</v>
+        <v>551</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>525</v>
+        <v>552</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>526</v>
+        <v>553</v>
       </c>
     </row>
     <row r="23" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>527</v>
+        <v>554</v>
       </c>
       <c r="B23" s="11">
         <v>46269.82745370371</v>
@@ -5407,30 +5809,30 @@
         <v>0.0033101851840910967</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>521</v>
+        <v>548</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>528</v>
+        <v>555</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>529</v>
+        <v>556</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>530</v>
+        <v>557</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>531</v>
+        <v>558</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>532</v>
+        <v>559</v>
       </c>
     </row>
     <row r="24" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>533</v>
+        <v>560</v>
       </c>
       <c r="B24" s="11">
         <v>46269.83311342592</v>
@@ -5446,16 +5848,16 @@
         <v>115</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>534</v>
+        <v>561</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>535</v>
+        <v>562</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>536</v>
+        <v>563</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>31</v>
@@ -5479,19 +5881,19 @@
         <v>0.03422453703751671</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>538</v>
+        <v>565</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>538</v>
+        <v>565</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>538</v>
+        <v>565</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>538</v>
+        <v>565</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>539</v>
+        <v>566</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
@@ -5511,25 +5913,25 @@
         <v>0.0005439814813144039</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>540</v>
+        <v>567</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>541</v>
+        <v>568</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>542</v>
+        <v>569</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>543</v>
+        <v>570</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>544</v>
+        <v>571</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>545</v>
+        <v>572</v>
       </c>
     </row>
     <row r="27" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5547,25 +5949,25 @@
         <v>0.0009375000008731149</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>546</v>
+        <v>573</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>547</v>
+        <v>574</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>548</v>
+        <v>575</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>549</v>
+        <v>576</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>550</v>
+        <v>577</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>551</v>
+        <v>578</v>
       </c>
     </row>
     <row r="28" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5583,25 +5985,25 @@
         <v>0.001574074074596865</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>552</v>
+        <v>579</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>553</v>
+        <v>580</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>554</v>
+        <v>581</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>555</v>
+        <v>582</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>556</v>
+        <v>583</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>557</v>
+        <v>584</v>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5654,19 +6056,19 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>558</v>
+        <v>585</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>558</v>
+        <v>585</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>558</v>
+        <v>585</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>558</v>
+        <v>585</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>559</v>
+        <v>586</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
@@ -5686,25 +6088,25 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>560</v>
+        <v>587</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>561</v>
+        <v>588</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>562</v>
+        <v>589</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>563</v>
+        <v>590</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>564</v>
+        <v>591</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>565</v>
+        <v>592</v>
       </c>
     </row>
     <row r="32" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5722,25 +6124,377 @@
         <v>0.0016319444439432118</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>566</v>
+        <v>593</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>567</v>
+        <v>594</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>568</v>
+        <v>595</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>569</v>
+        <v>596</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>570</v>
+        <v>597</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>571</v>
+        <v>598</v>
+      </c>
+    </row>
+    <row r="33" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="7" t="s">
+        <v>285</v>
+      </c>
+      <c r="B33" s="8">
+        <v>46270.44430555556</v>
+      </c>
+      <c r="C33" s="8">
+        <v>46270.45391203703</v>
+      </c>
+      <c r="D33" s="9">
+        <f>C33-B33</f>
+        <v>0.009606481482478557</v>
+      </c>
+      <c r="E33" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="H33" s="7" t="s">
+        <v>599</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>600</v>
+      </c>
+      <c r="J33" s="7"/>
+      <c r="K33" s="7"/>
+    </row>
+    <row r="34" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
+        <v>288</v>
+      </c>
+      <c r="B34" s="11">
+        <v>46270.44818287037</v>
+      </c>
+      <c r="C34" s="11">
+        <v>46270.44961805556</v>
+      </c>
+      <c r="D34" s="12">
+        <f>C34-B34</f>
+        <v>0.0014351851859828457</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>602</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>603</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="35" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>295</v>
+      </c>
+      <c r="B35" s="11">
+        <v>46270.449108796296</v>
+      </c>
+      <c r="C35" s="11">
+        <v>46270.44961805556</v>
+      </c>
+      <c r="D35" s="12">
+        <f>C35-B35</f>
+        <v>0.0005092592582514044</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>608</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>611</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="7" t="s">
+        <v>346</v>
+      </c>
+      <c r="B36" s="8">
+        <v>46270.46361111111</v>
+      </c>
+      <c r="C36" s="8">
+        <v>46270.47930555556</v>
+      </c>
+      <c r="D36" s="9">
+        <f>C36-B36</f>
+        <v>0.015694444446126</v>
+      </c>
+      <c r="E36" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="G36" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="H36" s="7" t="s">
+        <v>613</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>614</v>
+      </c>
+      <c r="J36" s="7"/>
+      <c r="K36" s="7"/>
+    </row>
+    <row r="37" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="B37" s="11">
+        <v>46270.465833333335</v>
+      </c>
+      <c r="C37" s="11">
+        <v>46270.46729166667</v>
+      </c>
+      <c r="D37" s="12">
+        <f>C37-B37</f>
+        <v>0.0014583333322661929</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>617</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>618</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>619</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K37" s="2" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="38" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
+        <v>621</v>
+      </c>
+      <c r="B38" s="11">
+        <v>46270.46697916667</v>
+      </c>
+      <c r="C38" s="11">
+        <v>46270.469942129625</v>
+      </c>
+      <c r="D38" s="12">
+        <f>C38-B38</f>
+        <v>0.0029629629643750377</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>622</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>623</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>625</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>626</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K38" s="2" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="39" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
+        <v>628</v>
+      </c>
+      <c r="B39" s="11">
+        <v>46270.46810185185</v>
+      </c>
+      <c r="C39" s="11">
+        <v>46270.46877314815</v>
+      </c>
+      <c r="D39" s="12">
+        <f>C39-B39</f>
+        <v>0.0006712962967867497</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>629</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>630</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>631</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>632</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>633</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="40" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
+        <v>635</v>
+      </c>
+      <c r="B40" s="11">
+        <v>46270.466782407406</v>
+      </c>
+      <c r="C40" s="11">
+        <v>46270.46729166667</v>
+      </c>
+      <c r="D40" s="12">
+        <f>C40-B40</f>
+        <v>0.0005092592582514044</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>636</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>637</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>638</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>639</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>640</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>627</v>
+      </c>
+    </row>
+    <row r="41" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" s="10" t="s">
+        <v>641</v>
+      </c>
+      <c r="B41" s="11">
+        <v>46270.471192129626</v>
+      </c>
+      <c r="C41" s="11">
+        <v>46270.47133101852</v>
+      </c>
+      <c r="D41" s="12">
+        <f>C41-B41</f>
+        <v>0.00013888888861401938</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>642</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>643</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>644</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>645</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="42" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
+        <v>646</v>
+      </c>
+      <c r="B42" s="11">
+        <v>46270.47395833333</v>
+      </c>
+      <c r="C42" s="11">
+        <v>46270.47930555556</v>
+      </c>
+      <c r="D42" s="12">
+        <f>C42-B42</f>
+        <v>0.005347222220734693</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>615</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>651</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(PersonFilter): improve row structure and accessibility
- Introduced ROW and ROW_NAME constants for consistent styling across options.
- Updated event handling to separate row selection and team expansion.
- Enhanced layout to ensure proper alignment and spacing of elements.
- Adjusted focus and hover states for better keyboard navigation and accessibility.
- Modified tests to reflect changes in component structure and behavior.
</commit_message>
<xml_diff>
--- a/Cowork changes 4 Sep 2026.xlsx
+++ b/Cowork changes 4 Sep 2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="872" uniqueCount="652">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="682">
   <si>
     <t>Cowork — changes, 4 September 2026</t>
   </si>
@@ -1113,6 +1113,96 @@
   </si>
   <si>
     <t>components/features/messages/TaskChatBrief.tsx</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>Whose tasks — the person dropdown</t>
+  </si>
+  <si>
+    <t>Requested: put the drop-down arrows on the right of each row, and open the sub-branch to the right instead of underneath the same row.</t>
+  </si>
+  <si>
+    <t>10a</t>
+  </si>
+  <si>
+    <t>Tasks ▸ toolbar ▸ the person dropdown (chief level only — it is a flat list lower down)</t>
+  </si>
+  <si>
+    <t>A team opens as its own column to the right, and its arrow moved to the right of the row</t>
+  </si>
+  <si>
+    <t>An indented accordion. The arrow sat on the LEFT of each name, and pressing it pushed that team in underneath, shoving every row below it down the list — so opening a branch to look at it moved the rows you had been reading out from under the pointer, and two branches open at different depths left you counting 14px of indent to work out who reported to whom.</t>
+  </si>
+  <si>
+    <t>The arrow sits at the right-hand end of the row, on the side the team appears on. Pressing it opens that team as its own panel beside the current one; the rows already on screen do not move. The chain of panels IS the reporting line, read left to right. Pressing an open arrow again closes that panel and everything to the right of it, and Escape steps back one panel at a time before closing the menu.</t>
+  </si>
+  <si>
+    <t>The state changed with the shape: a PATH of open managers rather than a set of expanded ids, because a set would let two managers at the same depth both claim the panel beside them. The panels are SIBLINGS in one strip rather than children of the panel that opened them — each panel scrolls its own overflow, so a panel rendered inside its parent would be cut off the moment that parent was long enough to need a scrollbar. Verified in a browser at 768px, where the third panel ran off the right of the screen: the strip now measures its own left edge and fits itself to what is left of the window, and scrolls the newest panel into view. Also removed a setState-in-effect that predates this change — opening onto the current selection is now done in the button's own handler, which is one render instead of two.</t>
+  </si>
+  <si>
+    <t>components/features/tasks/PersonFilter.tsx; personFilterWiring.test.ts (5 new checks); lib/help/knowledge.ts (“What does All members mean?”)</t>
+  </si>
+  <si>
+    <t>10b</t>
+  </si>
+  <si>
+    <t>Tasks ▸ the person dropdown ▸ All members</t>
+  </si>
+  <si>
+    <t>All members is the same width as the names under it</t>
+  </si>
+  <si>
+    <t>It ran the full width of the panel while every name below it stopped 26px short — the names sit beside a reserved slot for the branch arrow and this row did not. So its highlight overhung theirs, and its count stood in a column of its own, 26px right of every other figure.</t>
+  </si>
+  <si>
+    <t>The same row frame as a name, arrow slot included. Measured in a browser: all four rows now 205px wide, ending at x=249, with every count’s right edge at x=239.</t>
+  </si>
+  <si>
+    <t>Nobody manages the whole company, so there is no arrow to put in that slot — but the slot is what makes the widths derive from one number instead of two. The same reason a leaf reserves it: a column whose rows are different lengths stops reading as a column. Pinned by a test that counts the spacers, so a third row added later cannot quietly go full-width.</t>
+  </si>
+  <si>
+    <t>components/features/tasks/PersonFilter.tsx; personFilterWiring.test.ts</t>
+  </si>
+  <si>
+    <t>10c</t>
+  </si>
+  <si>
+    <t>Tasks ▸ the person dropdown ▸ every row</t>
+  </si>
+  <si>
+    <t>Rows fill the panel, and the arrow sits on top of them</t>
+  </si>
+  <si>
+    <t>10b lined the counts up by giving every row a 24px spacer beside the name — which fixed the counts and broke the rows. A spacer is an ELEMENT: it takes width from the row, so every highlight stopped 27px short of the panel's right edge while starting 1px from its left. Measured: rows 45..249 inside a panel whose inner edges are 44 and 276. A lopsided highlight is what the eye reads as a wrong width, which is what the owner was pointing at both times.</t>
+  </si>
+  <si>
+    <t>One shared row frame, `w-full` with `pr-9`. The reserved space moved out of a spacer element and into the row's own padding, so it still holds the counts in one column but no longer shortens anything. The arrow is absolutely positioned ON that padding. Measured after: every row 45..275 against inner edges of 44 and 276 — 1px each side — and every count's right edge at 239, in both panels.</t>
+  </si>
+  <si>
+    <t>Third attempt, and the first two failed the same way: I fixed the property that was named and broke the one beside it. Padding rather than a spacer is what lets both hold at once — the row keeps its full width AND the counts keep their column, from one number instead of two. The arrow stays a SIBLING of the name button, absolutely placed, because a button inside a button is invalid HTML that browsers flatten. The hover moved onto a wrapping `group` at the same time: with the arrow sitting on the row, a bare hover on the name would have dropped the highlight the moment the pointer crossed onto the arrow. Measured over the arrow — row rgba(255,255,255,0.08), arrow rgba(255,255,255,0.18).</t>
+  </si>
+  <si>
+    <t>components/features/tasks/PersonFilter.tsx; personFilterWiring.test.ts (4 checks replacing the spacer ones)</t>
+  </si>
+  <si>
+    <t>10d</t>
+  </si>
+  <si>
+    <t>The row fill moved onto the wrapper, which is how the rest of the app does it</t>
+  </si>
+  <si>
+    <t>10c reached a full-width row by making the name button `w-full pr-9` and hanging the arrow off it absolutely. The geometry was right, but the mechanism was borrowed from this codebase’s INPUT idiom — PasswordInput.tsx and the three form fields that copy it — and every one of those is an `&lt;input&gt;`, a surface that has to own its own background and therefore cannot hand it to a parent. No list row in the repo does it. It also coupled three numbers by hand (`pr-9`, `right-1`, `h-6 w-6`) with nothing to catch a drift between them, and it gave the row NO focus state at all: tabbing through the menu lit nothing, because `group-hover:` only covers a pointer.</t>
+  </si>
+  <si>
+    <t>The wash, the radius and the side padding sit on the non-pressable wrapper; the name button and the arrow are ordinary flex siblings inside it; a leaf reserves the arrow’s box with a spacer again. Identical geometry — rows 45..275 against inner edges of 44 and 276, counts at 239 — with no absolute positioning and no magic numbers, since the arrow’s own box IS the reservation. `focus-within` on the wrapper and `focus-visible` on the arrow give the menu a keyboard state it did not have.</t>
+  </si>
+  <si>
+    <t>The spacer was never the problem. The wash being on the BUTTON was — that is what let a 24px sibling take width off the highlighted surface, and it is the thing all three earlier attempts missed while arguing about the spacer. Found by fanning four readers across every menu, tree and trailing control in the app rather than guessing a fourth time: the rule is written down at TaskTable.tsx:1358 (padding moved off the row into the cells “so the hover wash still reaches the panel’s edges”), four files spend a negative margin to buy it back, and roughly twenty rows already put the fill on a wrapper — MindMapOutline.tsx’s tree row being the closest twin. `group-hover:` driving a row’s own fill existed in exactly one file in the repo: this one.</t>
+  </si>
+  <si>
+    <t>components/features/tasks/PersonFilter.tsx; personFilterWiring.test.ts (4 checks rewritten)</t>
   </si>
   <si>
     <t>What is open</t>
@@ -2664,7 +2754,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K56"/>
+  <dimension ref="A1:K61"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -3390,11 +3480,11 @@
         <v>46269.747210648144</v>
       </c>
       <c r="C22" s="8">
-        <v>46270.51725694444</v>
+        <v>46269.76292824074</v>
       </c>
       <c r="D22" s="9">
         <f>C22-B22</f>
-        <v>0.7700462962962963</v>
+        <v>0.015717592592592592</v>
       </c>
       <c r="E22" s="7" t="s">
         <v>167</v>
@@ -3524,11 +3614,11 @@
         <v>46269.773148148146</v>
       </c>
       <c r="C26" s="8">
-        <v>46270.51725694444</v>
+        <v>46269.84722222222</v>
       </c>
       <c r="D26" s="9">
         <f>C26-B26</f>
-        <v>0.7441087962962963</v>
+        <v>0.07407407407407407</v>
       </c>
       <c r="E26" s="7" t="s">
         <v>190</v>
@@ -3694,11 +3784,11 @@
         <v>46269.79305555555</v>
       </c>
       <c r="C31" s="11">
-        <v>46270.51725694444</v>
+        <v>46269.810069444444</v>
       </c>
       <c r="D31" s="12">
         <f>C31-B31</f>
-        <v>0.7242013888888889</v>
+        <v>0.017013888888888887</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>219</v>
@@ -3802,11 +3892,11 @@
         <v>46269.82777777778</v>
       </c>
       <c r="C34" s="11">
-        <v>46270.51725694444</v>
+        <v>46269.834027777775</v>
       </c>
       <c r="D34" s="12">
         <f>C34-B34</f>
-        <v>0.6894791666666666</v>
+        <v>0.00625</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>115</v>
@@ -3874,11 +3964,11 @@
         <v>46269.83541666667</v>
       </c>
       <c r="C36" s="11">
-        <v>46270.51725694444</v>
+        <v>46269.84722222222</v>
       </c>
       <c r="D36" s="12">
         <f>C36-B36</f>
-        <v>0.6818402777777778</v>
+        <v>0.011805555555555555</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>252</v>
@@ -4008,11 +4098,11 @@
         <v>46269.84722222222</v>
       </c>
       <c r="C40" s="11">
-        <v>46270.51725694444</v>
+        <v>46269.878437499996</v>
       </c>
       <c r="D40" s="12">
         <f>C40-B40</f>
-        <v>0.6700347222222223</v>
+        <v>0.03121527777777778</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>273</v>
@@ -4080,11 +4170,11 @@
         <v>46269.813368055555</v>
       </c>
       <c r="C42" s="8">
-        <v>46270.51725694444</v>
+        <v>46270.447222222225</v>
       </c>
       <c r="D42" s="9">
         <f>C42-B42</f>
-        <v>0.7038888888888889</v>
+        <v>0.6338541666666667</v>
       </c>
       <c r="E42" s="7" t="s">
         <v>286</v>
@@ -4265,11 +4355,11 @@
         <v>46270.51388888889</v>
       </c>
       <c r="C48" s="11">
-        <v>46270.51725694444</v>
+        <v>46270.51944444445</v>
       </c>
       <c r="D48" s="12">
         <f>C48-B48</f>
-        <v>0.0033680555555555556</v>
+        <v>0.005555555555555556</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>315</v>
@@ -4337,11 +4427,11 @@
         <v>46270.43513888889</v>
       </c>
       <c r="C50" s="11">
-        <v>46270.51725694444</v>
+        <v>46270.43833333333</v>
       </c>
       <c r="D50" s="12">
         <f>C50-B50</f>
-        <v>0.08211805555555556</v>
+        <v>0.0031944444444444446</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>161</v>
@@ -4409,11 +4499,11 @@
         <v>46270.43833333333</v>
       </c>
       <c r="C52" s="11">
-        <v>46270.51725694444</v>
+        <v>46270.447222222225</v>
       </c>
       <c r="D52" s="12">
         <f>C52-B52</f>
-        <v>0.07892361111111111</v>
+        <v>0.008888888888888889</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>340</v>
@@ -4561,9 +4651,179 @@
         <v>365</v>
       </c>
     </row>
+    <row r="57" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="B57" s="8">
+        <v>46270.52013888889</v>
+      </c>
+      <c r="C57" s="8">
+        <v>46270.55626157408</v>
+      </c>
+      <c r="D57" s="9">
+        <f>C57-B57</f>
+        <v>0.03612268518518519</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="J57" s="7"/>
+      <c r="K57" s="7"/>
+    </row>
+    <row r="58" ht="258" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" s="10" t="s">
+        <v>369</v>
+      </c>
+      <c r="B58" s="11">
+        <v>46270.52013888889</v>
+      </c>
+      <c r="C58" s="11">
+        <v>46270.53611111111</v>
+      </c>
+      <c r="D58" s="12">
+        <f>C58-B58</f>
+        <v>0.01597222222222222</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K58" s="2" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="59" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="B59" s="11">
+        <v>46270.5375</v>
+      </c>
+      <c r="C59" s="11">
+        <v>46270.54166666667</v>
+      </c>
+      <c r="D59" s="12">
+        <f>C59-B59</f>
+        <v>0.004166666666666667</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>377</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>379</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>380</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>381</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K59" s="2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="60" ht="230" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="B60" s="11">
+        <v>46270.54236111111</v>
+      </c>
+      <c r="C60" s="11">
+        <v>46270.54791666666</v>
+      </c>
+      <c r="D60" s="12">
+        <f>C60-B60</f>
+        <v>0.005555555555555556</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>385</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>386</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="I60" s="2" t="s">
+        <v>388</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K60" s="2" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="61" ht="244" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="B61" s="11">
+        <v>46270.54791666666</v>
+      </c>
+      <c r="C61" s="11">
+        <v>46270.55626157408</v>
+      </c>
+      <c r="D61" s="12">
+        <f>C61-B61</f>
+        <v>0.008344907407407407</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>384</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>391</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K61" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K56"/>
-  <mergeCells count="11">
+  <autoFilter ref="A1:K61"/>
+  <mergeCells count="12">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="E14:H14"/>
@@ -4575,6 +4835,7 @@
     <mergeCell ref="A47:K47"/>
     <mergeCell ref="E53:H53"/>
     <mergeCell ref="E55:H55"/>
+    <mergeCell ref="E57:H57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4596,13 +4857,13 @@
         <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>366</v>
+        <v>396</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>367</v>
+        <v>397</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>368</v>
+        <v>398</v>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4610,27 +4871,27 @@
         <v>137</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>371</v>
+        <v>401</v>
       </c>
     </row>
     <row r="3" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>372</v>
+        <v>402</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>373</v>
+        <v>403</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>374</v>
+        <v>404</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>375</v>
+        <v>405</v>
       </c>
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4638,13 +4899,13 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>376</v>
+        <v>406</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>377</v>
+        <v>407</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>378</v>
+        <v>408</v>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4652,13 +4913,13 @@
         <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>379</v>
+        <v>409</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>381</v>
+        <v>411</v>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4666,13 +4927,13 @@
         <v>108</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>382</v>
+        <v>412</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>383</v>
+        <v>413</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>384</v>
+        <v>414</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4680,13 +4941,13 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>385</v>
+        <v>415</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>386</v>
+        <v>416</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4694,27 +4955,27 @@
         <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>389</v>
+        <v>419</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>390</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>391</v>
+        <v>421</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>392</v>
+        <v>422</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>393</v>
+        <v>423</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>394</v>
+        <v>424</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4722,13 +4983,13 @@
         <v>251</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>395</v>
+        <v>425</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>396</v>
+        <v>426</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>397</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4736,13 +4997,13 @@
         <v>199</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>398</v>
+        <v>428</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>400</v>
+        <v>430</v>
       </c>
     </row>
     <row r="12" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4750,13 +5011,13 @@
         <v>199</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>401</v>
+        <v>431</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>402</v>
+        <v>432</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>403</v>
+        <v>433</v>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4764,27 +5025,27 @@
         <v>199</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>404</v>
+        <v>434</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>405</v>
+        <v>435</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>406</v>
+        <v>436</v>
       </c>
     </row>
     <row r="14" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>407</v>
+        <v>437</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>408</v>
+        <v>438</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>409</v>
+        <v>439</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>410</v>
+        <v>440</v>
       </c>
     </row>
   </sheetData>
@@ -4807,7 +5068,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>411</v>
+        <v>441</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -4820,179 +5081,179 @@
         <v>40</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>412</v>
+        <v>442</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>413</v>
+        <v>443</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>414</v>
+        <v>444</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>415</v>
+        <v>445</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>416</v>
+        <v>446</v>
       </c>
     </row>
     <row r="3" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>417</v>
+        <v>447</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>418</v>
+        <v>448</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>419</v>
+        <v>449</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="4" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>423</v>
+        <v>453</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>424</v>
+        <v>454</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>425</v>
+        <v>455</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>426</v>
+        <v>456</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>428</v>
+        <v>458</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>429</v>
+        <v>459</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>430</v>
+        <v>460</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>431</v>
+        <v>461</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>432</v>
+        <v>462</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>433</v>
+        <v>463</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>434</v>
+        <v>464</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>435</v>
+        <v>465</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>436</v>
+        <v>466</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>437</v>
+        <v>467</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>438</v>
+        <v>468</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="8" ht="92" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>439</v>
+        <v>469</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>440</v>
+        <v>470</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>441</v>
+        <v>471</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>442</v>
+        <v>472</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>443</v>
+        <v>473</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>444</v>
+        <v>474</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>445</v>
+        <v>475</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>446</v>
+        <v>476</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>447</v>
+        <v>477</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>448</v>
+        <v>478</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>449</v>
+        <v>479</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>451</v>
+        <v>481</v>
       </c>
       <c r="E10" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="F10" s="13" t="s">
         <v>452</v>
-      </c>
-      <c r="F10" s="13" t="s">
-        <v>422</v>
       </c>
     </row>
   </sheetData>
@@ -5117,7 +5378,7 @@
         <v>322</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>453</v>
+        <v>483</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -5140,22 +5401,22 @@
         <v>159</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>454</v>
+        <v>484</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>455</v>
+        <v>485</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>456</v>
+        <v>486</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>457</v>
+        <v>487</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>458</v>
+        <v>488</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5173,19 +5434,19 @@
         <v>0.017418981482478557</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>459</v>
+        <v>489</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>459</v>
+        <v>489</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>459</v>
+        <v>489</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>459</v>
+        <v>489</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>460</v>
+        <v>490</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -5205,25 +5466,25 @@
         <v>0.0020370370366435964</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>461</v>
+        <v>491</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>462</v>
+        <v>492</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>463</v>
+        <v>493</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>464</v>
+        <v>494</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>465</v>
+        <v>495</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>466</v>
+        <v>496</v>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5241,25 +5502,25 @@
         <v>0.0026504629640839994</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>467</v>
+        <v>497</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>468</v>
+        <v>498</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>469</v>
+        <v>499</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>470</v>
+        <v>500</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>471</v>
+        <v>501</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>472</v>
+        <v>502</v>
       </c>
     </row>
     <row r="8" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5277,25 +5538,25 @@
         <v>0.00010416666555101983</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>473</v>
+        <v>503</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>474</v>
+        <v>504</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>475</v>
+        <v>505</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>476</v>
+        <v>506</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>477</v>
+        <v>507</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>478</v>
+        <v>508</v>
       </c>
     </row>
     <row r="9" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5313,30 +5574,30 @@
         <v>0.00028935185036971234</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>479</v>
+        <v>509</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>480</v>
+        <v>510</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>481</v>
+        <v>511</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>482</v>
+        <v>512</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>483</v>
+        <v>513</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>484</v>
+        <v>514</v>
       </c>
     </row>
     <row r="10" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>485</v>
+        <v>515</v>
       </c>
       <c r="B10" s="11">
         <v>46269.77627314815</v>
@@ -5352,27 +5613,27 @@
         <v>115</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>486</v>
+        <v>516</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>487</v>
+        <v>517</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>488</v>
+        <v>518</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>489</v>
+        <v>519</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>490</v>
+        <v>520</v>
       </c>
     </row>
     <row r="11" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>491</v>
+        <v>521</v>
       </c>
       <c r="B11" s="11">
         <v>46269.78513888889</v>
@@ -5385,30 +5646,30 @@
         <v>0.0005555555544560775</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>492</v>
+        <v>522</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>493</v>
+        <v>523</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>494</v>
+        <v>524</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>495</v>
+        <v>525</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>496</v>
+        <v>526</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>484</v>
+        <v>514</v>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>497</v>
+        <v>527</v>
       </c>
       <c r="B12" s="11">
         <v>46269.784733796296</v>
@@ -5421,30 +5682,30 @@
         <v>0.0009606481471564621</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>498</v>
+        <v>528</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>499</v>
+        <v>529</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>500</v>
+        <v>530</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>501</v>
+        <v>531</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>502</v>
+        <v>532</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>503</v>
+        <v>533</v>
       </c>
     </row>
     <row r="13" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>504</v>
+        <v>534</v>
       </c>
       <c r="B13" s="11">
         <v>46269.78622685185</v>
@@ -5460,16 +5721,16 @@
         <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>505</v>
+        <v>535</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>506</v>
+        <v>536</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>507</v>
+        <v>537</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>508</v>
+        <v>538</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>31</v>
@@ -5493,19 +5754,19 @@
         <v>0.0065393518525525</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>509</v>
+        <v>539</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>509</v>
+        <v>539</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>509</v>
+        <v>539</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>509</v>
+        <v>539</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>510</v>
+        <v>540</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -5525,25 +5786,25 @@
         <v>0.00020833333474001847</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>511</v>
+        <v>541</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>512</v>
+        <v>542</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>513</v>
+        <v>543</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>514</v>
+        <v>544</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>515</v>
+        <v>545</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>516</v>
+        <v>546</v>
       </c>
     </row>
     <row r="16" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5561,25 +5822,25 @@
         <v>0.0016666666670062114</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>517</v>
+        <v>547</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>518</v>
+        <v>548</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>519</v>
+        <v>549</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>520</v>
+        <v>550</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>521</v>
+        <v>551</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>522</v>
+        <v>552</v>
       </c>
     </row>
     <row r="17" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5600,16 +5861,16 @@
         <v>115</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>523</v>
+        <v>553</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>524</v>
+        <v>554</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>525</v>
+        <v>555</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>526</v>
+        <v>556</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>31</v>
@@ -5633,19 +5894,19 @@
         <v>0.01622685185066075</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>527</v>
+        <v>557</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>528</v>
+        <v>558</v>
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -5665,25 +5926,25 @@
         <v>0.0001851851848186925</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>529</v>
+        <v>559</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>530</v>
+        <v>560</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>531</v>
+        <v>561</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>532</v>
+        <v>562</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>533</v>
+        <v>563</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>534</v>
+        <v>564</v>
       </c>
     </row>
     <row r="20" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5701,25 +5962,25 @@
         <v>0.0015509259246755391</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>535</v>
+        <v>565</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>536</v>
+        <v>566</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>537</v>
+        <v>567</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>538</v>
+        <v>568</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>539</v>
+        <v>569</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>540</v>
+        <v>570</v>
       </c>
     </row>
     <row r="21" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5737,30 +5998,30 @@
         <v>0.001701388890069211</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>541</v>
+        <v>571</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>542</v>
+        <v>572</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>543</v>
+        <v>573</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>544</v>
+        <v>574</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>545</v>
+        <v>575</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>546</v>
+        <v>576</v>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>547</v>
+        <v>577</v>
       </c>
       <c r="B22" s="11">
         <v>46269.82821759259</v>
@@ -5773,30 +6034,30 @@
         <v>0.0010532407395658083</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>548</v>
+        <v>578</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>549</v>
+        <v>579</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>550</v>
+        <v>580</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>551</v>
+        <v>581</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>552</v>
+        <v>582</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>553</v>
+        <v>583</v>
       </c>
     </row>
     <row r="23" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>554</v>
+        <v>584</v>
       </c>
       <c r="B23" s="11">
         <v>46269.82745370371</v>
@@ -5809,30 +6070,30 @@
         <v>0.0033101851840910967</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>548</v>
+        <v>578</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>555</v>
+        <v>585</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>556</v>
+        <v>586</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>557</v>
+        <v>587</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>558</v>
+        <v>588</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>559</v>
+        <v>589</v>
       </c>
     </row>
     <row r="24" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>560</v>
+        <v>590</v>
       </c>
       <c r="B24" s="11">
         <v>46269.83311342592</v>
@@ -5848,16 +6109,16 @@
         <v>115</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>561</v>
+        <v>591</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>562</v>
+        <v>592</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>563</v>
+        <v>593</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>564</v>
+        <v>594</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>31</v>
@@ -5881,19 +6142,19 @@
         <v>0.03422453703751671</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>565</v>
+        <v>595</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>565</v>
+        <v>595</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>565</v>
+        <v>595</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>565</v>
+        <v>595</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>566</v>
+        <v>596</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
@@ -5913,25 +6174,25 @@
         <v>0.0005439814813144039</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>567</v>
+        <v>597</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>568</v>
+        <v>598</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>569</v>
+        <v>599</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>570</v>
+        <v>600</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>571</v>
+        <v>601</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>572</v>
+        <v>602</v>
       </c>
     </row>
     <row r="27" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5949,25 +6210,25 @@
         <v>0.0009375000008731149</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>573</v>
+        <v>603</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>574</v>
+        <v>604</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>575</v>
+        <v>605</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>576</v>
+        <v>606</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>577</v>
+        <v>607</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>578</v>
+        <v>608</v>
       </c>
     </row>
     <row r="28" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5985,25 +6246,25 @@
         <v>0.001574074074596865</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>579</v>
+        <v>609</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>580</v>
+        <v>610</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>581</v>
+        <v>611</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>582</v>
+        <v>612</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>583</v>
+        <v>613</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>584</v>
+        <v>614</v>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6056,19 +6317,19 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>585</v>
+        <v>615</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>585</v>
+        <v>615</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>585</v>
+        <v>615</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>585</v>
+        <v>615</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>586</v>
+        <v>616</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
@@ -6088,25 +6349,25 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>587</v>
+        <v>617</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>588</v>
+        <v>618</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>589</v>
+        <v>619</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>590</v>
+        <v>620</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>591</v>
+        <v>621</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>592</v>
+        <v>622</v>
       </c>
     </row>
     <row r="32" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6124,25 +6385,25 @@
         <v>0.0016319444439432118</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>593</v>
+        <v>623</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>594</v>
+        <v>624</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>595</v>
+        <v>625</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>596</v>
+        <v>626</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>597</v>
+        <v>627</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>598</v>
+        <v>628</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6160,19 +6421,19 @@
         <v>0.009606481482478557</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>599</v>
+        <v>629</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>599</v>
+        <v>629</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>599</v>
+        <v>629</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>599</v>
+        <v>629</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>600</v>
+        <v>630</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -6192,25 +6453,25 @@
         <v>0.0014351851859828457</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>601</v>
+        <v>631</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>602</v>
+        <v>632</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>603</v>
+        <v>633</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>604</v>
+        <v>634</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>605</v>
+        <v>635</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>606</v>
+        <v>636</v>
       </c>
     </row>
     <row r="35" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6228,25 +6489,25 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>607</v>
+        <v>637</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>608</v>
+        <v>638</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>609</v>
+        <v>639</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>610</v>
+        <v>640</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>611</v>
+        <v>641</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>612</v>
+        <v>642</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6264,19 +6525,19 @@
         <v>0.015694444446126</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>613</v>
+        <v>643</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>613</v>
+        <v>643</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>613</v>
+        <v>643</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>613</v>
+        <v>643</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>614</v>
+        <v>644</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
@@ -6296,30 +6557,30 @@
         <v>0.0014583333322661929</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>615</v>
+        <v>645</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>616</v>
+        <v>646</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>617</v>
+        <v>647</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>618</v>
+        <v>648</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>619</v>
+        <v>649</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>620</v>
+        <v>650</v>
       </c>
     </row>
     <row r="38" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>621</v>
+        <v>651</v>
       </c>
       <c r="B38" s="11">
         <v>46270.46697916667</v>
@@ -6332,30 +6593,30 @@
         <v>0.0029629629643750377</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>622</v>
+        <v>652</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>623</v>
+        <v>653</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>624</v>
+        <v>654</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>625</v>
+        <v>655</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>626</v>
+        <v>656</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>627</v>
+        <v>657</v>
       </c>
     </row>
     <row r="39" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>628</v>
+        <v>658</v>
       </c>
       <c r="B39" s="11">
         <v>46270.46810185185</v>
@@ -6368,30 +6629,30 @@
         <v>0.0006712962967867497</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>629</v>
+        <v>659</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>630</v>
+        <v>660</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>631</v>
+        <v>661</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>632</v>
+        <v>662</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>633</v>
+        <v>663</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>634</v>
+        <v>664</v>
       </c>
     </row>
     <row r="40" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>635</v>
+        <v>665</v>
       </c>
       <c r="B40" s="11">
         <v>46270.466782407406</v>
@@ -6404,30 +6665,30 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>636</v>
+        <v>666</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>637</v>
+        <v>667</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>638</v>
+        <v>668</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>639</v>
+        <v>669</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>640</v>
+        <v>670</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>627</v>
+        <v>657</v>
       </c>
     </row>
     <row r="41" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>641</v>
+        <v>671</v>
       </c>
       <c r="B41" s="11">
         <v>46270.471192129626</v>
@@ -6443,16 +6704,16 @@
         <v>115</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>642</v>
+        <v>672</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>643</v>
+        <v>673</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>644</v>
+        <v>674</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>645</v>
+        <v>675</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>31</v>
@@ -6463,7 +6724,7 @@
     </row>
     <row r="42" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>646</v>
+        <v>676</v>
       </c>
       <c r="B42" s="11">
         <v>46270.47395833333</v>
@@ -6476,25 +6737,25 @@
         <v>0.005347222220734693</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>615</v>
+        <v>645</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>647</v>
+        <v>677</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>648</v>
+        <v>678</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>649</v>
+        <v>679</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>650</v>
+        <v>680</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>651</v>
+        <v>681</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add image handling features and tests for spreadsheet component
- Implemented image insertion functionality in the spreadsheet, including tests for image import, resizing, and rendering.
- Created utility functions for managing image crops and rotations.
- Added tests for branch column positioning logic to ensure proper alignment in UI.
- Established limits for image dimensions during import to maintain layout integrity.
- Ensured that images are handled efficiently without unnecessary quality loss during processing.
</commit_message>
<xml_diff>
--- a/Cowork changes 4 Sep 2026.xlsx
+++ b/Cowork changes 4 Sep 2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="682">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="712">
   <si>
     <t>Cowork — changes, 4 September 2026</t>
   </si>
@@ -1205,6 +1205,57 @@
     <t>components/features/tasks/PersonFilter.tsx; personFilterWiring.test.ts (4 checks rewritten)</t>
   </si>
   <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>A picture in a cell</t>
+  </si>
+  <si>
+    <t>Requested: an Insert ▸ Image entry on the right-click menu, the picture stored to Drive, an editor on import to crop, rotate and size it, the cell sized from the picture, and a maximum size enforced on import only — not on resizing the cell afterwards.</t>
+  </si>
+  <si>
+    <t>11a</t>
+  </si>
+  <si>
+    <t>Sheets ▸ right-click a cell ▸ Insert ▸ Image</t>
+  </si>
+  <si>
+    <t>Insert ▸ Image, with a crop-and-rotate editor, sizing the cell from the picture</t>
+  </si>
+  <si>
+    <t>The ribbon’s Insert tab already had an Image button that uploaded to Drive and wrote =IMAGE(url) — so the store was settled and working. Three things were missing: it was not on the right-click menu at all, there was no editor between choosing a file and it landing, and the cell was left at its default 100 × 24 whatever the picture’s size, which for a photograph is a smudge. The help article still said pictures “have nowhere to live, because a cell holds a value, its formatting and an optional link and nothing else”.</t>
+  </si>
+  <si>
+    <t>Insert ▸ Image sits under Insert beside Row above and Column left. Choosing a file opens an editor: drag the corners to crop, Rotate left / Rotate right, and a line that names the size the cell will become. Insert uploads the edited picture to Drive — the same store documents and mind-map cards use — and writes it into the cell, sizing the row and column to the picture. The ceiling on import is 480 × 360: anything larger is scaled down keeping its proportions and the editor says so with both sizes. Past that the cell is an ordinary cell and can be dragged to any size, which is exactly the distinction asked for.</t>
+  </si>
+  <si>
+    <t>Three pure modules first, proven at a terminal before any of it was drawn: the import clamp (11 tests), the crop-and-rotation arithmetic (16), and then the wiring (17). The bytes are re-encoded at the size the cell will show — a 4000px photograph otherwise goes through Drive, down the wire and into every future load of the sheet to be thrown away by the browser — but a picture nobody edited and that needs no shrinking is uploaded untouched, because re-encoding a JPEG for no change costs a generation of quality. Verified in a browser with a 1200 × 400 probe image carrying a different colour in each corner: one clockwise turn moved red from top-left to top-right and produced a 120 × 360 file, and a dragged crop produced 480 × 187 with red the only marker left in it.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/{ImageImportDialog,FilePicker,SpreadsheetGrid,useSpreadsheet,CellVisual}.tsx; lib/spreadsheet/{imageImport,imageEdit,imageCanvas}.ts; components/ui/DriveImage.tsx; lib/help/knowledge.ts (“The Insert tab in a sheet”)</t>
+  </si>
+  <si>
+    <t>11b</t>
+  </si>
+  <si>
+    <t>Sheets ▸ a cell holding a picture</t>
+  </si>
+  <si>
+    <t>Two defects found by a codebase review, before either shipped</t>
+  </si>
+  <si>
+    <t>First: the cell was resized BEFORE the formula was written, and the write is gated twice more than the resize is — by data validation and by protection on a RANGE, neither of which `applyStructural` checks. Inserting a picture into a validated or protected cell would have left it resized to a picture that was never allowed in, with nothing said. Second: a picture in a cell was drawn by a bare &lt;img&gt; with one source, and a file uploaded a second ago 404s on Google’s CDN until it is indexed — so the cell would have been broken at exactly the moment somebody had just filled it.</t>
+  </si>
+  <si>
+    <t>Both gates now answer before either half runs, so a refused cell is not resized on the way to being refused, and the refusal names the rule. The picture renders through `DriveImage`, which walks CDN → proxy → the stored address as each fails, and recovers the Drive id from the URL itself; a hand-typed https address that is not a Drive file still passes straight through as its own only source.</t>
+  </si>
+  <si>
+    <t>Neither was visible from the feature’s own code, and neither would have shown up in the browser test I ran — the upload path needs a signed-in account and the protection path needs a protected sheet. Found by fanning six readers across the context menu, the cell model, the render path, persistence, storage and the dialog conventions, then having one agent write the plan from what they returned. The same review confirmed the two architectural choices already made: reuse `uploadDriveFile` rather than build storage, and keep the picture in the cell VALUE as =IMAGE(…) rather than add a `Worksheet.images` map — which would have had to be threaded through eight places with five points that silently drop it, including the 10-second local-file re-import.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/{useSpreadsheet,CellVisual}.tsx; components/ui/DriveImage.tsx</t>
+  </si>
+  <si>
     <t>What is open</t>
   </si>
   <si>
@@ -2061,6 +2112,45 @@
   </si>
   <si>
     <t>lib/rules/sheets/leaveGuard.ts (+5 tests); Spreadsheet.tsx; lib/help/knowledge.ts</t>
+  </si>
+  <si>
+    <t>Where a team's column sits in the person picker</t>
+  </si>
+  <si>
+    <t>Reported: opening somebody's team put their people at the top of the panel rather than beside the person they report to.</t>
+  </si>
+  <si>
+    <t>Tasks ▸ the person picker</t>
+  </si>
+  <si>
+    <t>A team's column starts level with its own row</t>
+  </si>
+  <si>
+    <t>Every column was top-aligned to the panel. Opening the team of somebody near the BOTTOM of a long list put their people up at the top, level with names they have nothing to do with and a whole list-height from the row that opened them — so the one thing the columns exist to show, who reports to whom, was the one thing the layout did not say.</t>
+  </si>
+  <si>
+    <t>The column starts level with the row it came from, and the chain reads as a staircase down and across. It slides back up only as far as it must to stay on screen, and never above the panel's own top.</t>
+  </si>
+  <si>
+    <t>Reported. Measured after paint rather than derived: the row's position depends on how many people are above it, how far its column is scrolled, and how far the column above was itself pushed down. Clamping is the part that can go wrong, so it is a tested rule rather than arithmetic in a component.</t>
+  </si>
+  <si>
+    <t>lib/rules/tasks/branchColumn.ts (new, 6 tests); PersonFilter.tsx; personFilterWiring.test.ts (+5)</t>
+  </si>
+  <si>
+    <t>9b</t>
+  </si>
+  <si>
+    <t>The article says where the column starts</t>
+  </si>
+  <si>
+    <t>It said the team opens 'as its own column to the right, beside them' — true of the intent, not of what was drawn.</t>
+  </si>
+  <si>
+    <t>It says the column starts level with that person's own row, and why that shape is the reporting line.</t>
+  </si>
+  <si>
+    <t>Project rule. The old wording was the one that made the defect hard to see: it described what everybody assumed was happening.</t>
   </si>
 </sst>
 </file>
@@ -2754,7 +2844,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K61"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -4659,11 +4749,11 @@
         <v>46270.52013888889</v>
       </c>
       <c r="C57" s="8">
-        <v>46270.55626157408</v>
+        <v>46270.62466435185</v>
       </c>
       <c r="D57" s="9">
         <f>C57-B57</f>
-        <v>0.03612268518518519</v>
+        <v>0.10452546296296296</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>367</v>
@@ -4793,11 +4883,11 @@
         <v>46270.54791666666</v>
       </c>
       <c r="C61" s="11">
-        <v>46270.55626157408</v>
+        <v>46270.55625</v>
       </c>
       <c r="D61" s="12">
         <f>C61-B61</f>
-        <v>0.008344907407407407</v>
+        <v>0.008333333333333333</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>384</v>
@@ -4821,9 +4911,107 @@
         <v>395</v>
       </c>
     </row>
+    <row r="62" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="B62" s="8">
+        <v>46270.55902777778</v>
+      </c>
+      <c r="C62" s="8">
+        <v>46270.62466435185</v>
+      </c>
+      <c r="D62" s="9">
+        <f>C62-B62</f>
+        <v>0.06563657407407407</v>
+      </c>
+      <c r="E62" s="7" t="s">
+        <v>397</v>
+      </c>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="J62" s="7"/>
+      <c r="K62" s="7"/>
+    </row>
+    <row r="63" ht="244" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" s="10" t="s">
+        <v>399</v>
+      </c>
+      <c r="B63" s="11">
+        <v>46270.55902777778</v>
+      </c>
+      <c r="C63" s="11">
+        <v>46270.62466435185</v>
+      </c>
+      <c r="D63" s="12">
+        <f>C63-B63</f>
+        <v>0.06563657407407407</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>403</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K63" s="2" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="64" ht="244" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" s="10" t="s">
+        <v>406</v>
+      </c>
+      <c r="B64" s="11">
+        <v>46270.61458333333</v>
+      </c>
+      <c r="C64" s="11">
+        <v>46270.62466435185</v>
+      </c>
+      <c r="D64" s="12">
+        <f>C64-B64</f>
+        <v>0.010081018518518519</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>411</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K64" s="2" t="s">
+        <v>412</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K61"/>
-  <mergeCells count="12">
+  <autoFilter ref="A1:K64"/>
+  <mergeCells count="13">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E3:H3"/>
     <mergeCell ref="E14:H14"/>
@@ -4836,6 +5024,7 @@
     <mergeCell ref="E53:H53"/>
     <mergeCell ref="E55:H55"/>
     <mergeCell ref="E57:H57"/>
+    <mergeCell ref="E62:H62"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -4857,13 +5046,13 @@
         <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>396</v>
+        <v>413</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>397</v>
+        <v>414</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>398</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4871,27 +5060,27 @@
         <v>137</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>399</v>
+        <v>416</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>400</v>
+        <v>417</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>401</v>
+        <v>418</v>
       </c>
     </row>
     <row r="3" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>402</v>
+        <v>419</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>403</v>
+        <v>420</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>404</v>
+        <v>421</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>405</v>
+        <v>422</v>
       </c>
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4899,13 +5088,13 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>406</v>
+        <v>423</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>407</v>
+        <v>424</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>408</v>
+        <v>425</v>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4913,13 +5102,13 @@
         <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>409</v>
+        <v>426</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>410</v>
+        <v>427</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>411</v>
+        <v>428</v>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4927,13 +5116,13 @@
         <v>108</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>412</v>
+        <v>429</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>413</v>
+        <v>430</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>414</v>
+        <v>431</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4941,13 +5130,13 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>415</v>
+        <v>432</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>416</v>
+        <v>433</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>417</v>
+        <v>434</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4955,27 +5144,27 @@
         <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>418</v>
+        <v>435</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>419</v>
+        <v>436</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>420</v>
+        <v>437</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>421</v>
+        <v>438</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>422</v>
+        <v>439</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>423</v>
+        <v>440</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>424</v>
+        <v>441</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4983,13 +5172,13 @@
         <v>251</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>425</v>
+        <v>442</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>426</v>
+        <v>443</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>427</v>
+        <v>444</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -4997,13 +5186,13 @@
         <v>199</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>428</v>
+        <v>445</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>429</v>
+        <v>446</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>430</v>
+        <v>447</v>
       </c>
     </row>
     <row r="12" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5011,13 +5200,13 @@
         <v>199</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>431</v>
+        <v>448</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>432</v>
+        <v>449</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>433</v>
+        <v>450</v>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5025,27 +5214,27 @@
         <v>199</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>434</v>
+        <v>451</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>435</v>
+        <v>452</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>436</v>
+        <v>453</v>
       </c>
     </row>
     <row r="14" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>437</v>
+        <v>454</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>438</v>
+        <v>455</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>439</v>
+        <v>456</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>440</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -5068,7 +5257,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>441</v>
+        <v>458</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -5081,179 +5270,179 @@
         <v>40</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>442</v>
+        <v>459</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>443</v>
+        <v>460</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>444</v>
+        <v>461</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>445</v>
+        <v>462</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>446</v>
+        <v>463</v>
       </c>
     </row>
     <row r="3" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>447</v>
+        <v>464</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>448</v>
+        <v>465</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>449</v>
+        <v>466</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>450</v>
+        <v>467</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>451</v>
+        <v>468</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="4" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>453</v>
+        <v>470</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>454</v>
+        <v>471</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>455</v>
+        <v>472</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>456</v>
+        <v>473</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>457</v>
+        <v>474</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>458</v>
+        <v>475</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>459</v>
+        <v>476</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>460</v>
+        <v>477</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>461</v>
+        <v>478</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>462</v>
+        <v>479</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>463</v>
+        <v>480</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>464</v>
+        <v>481</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>465</v>
+        <v>482</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>466</v>
+        <v>483</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>467</v>
+        <v>484</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>468</v>
+        <v>485</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" ht="92" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>469</v>
+        <v>486</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>470</v>
+        <v>487</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>471</v>
+        <v>488</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>472</v>
+        <v>489</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>473</v>
+        <v>490</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>474</v>
+        <v>491</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>475</v>
+        <v>492</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>476</v>
+        <v>493</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>477</v>
+        <v>494</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>478</v>
+        <v>495</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>479</v>
+        <v>496</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>480</v>
+        <v>497</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>481</v>
+        <v>498</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>482</v>
+        <v>499</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>452</v>
+        <v>469</v>
       </c>
     </row>
   </sheetData>
@@ -5267,7 +5456,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K45"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -5378,7 +5567,7 @@
         <v>322</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>483</v>
+        <v>500</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -5401,22 +5590,22 @@
         <v>159</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>484</v>
+        <v>501</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>485</v>
+        <v>502</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>486</v>
+        <v>503</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>487</v>
+        <v>504</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>488</v>
+        <v>505</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5434,19 +5623,19 @@
         <v>0.017418981482478557</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>489</v>
+        <v>506</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>490</v>
+        <v>507</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -5466,25 +5655,25 @@
         <v>0.0020370370366435964</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>491</v>
+        <v>508</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>492</v>
+        <v>509</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>493</v>
+        <v>510</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>494</v>
+        <v>511</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>495</v>
+        <v>512</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>496</v>
+        <v>513</v>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5502,25 +5691,25 @@
         <v>0.0026504629640839994</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>497</v>
+        <v>514</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>498</v>
+        <v>515</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>499</v>
+        <v>516</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>500</v>
+        <v>517</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>501</v>
+        <v>518</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>502</v>
+        <v>519</v>
       </c>
     </row>
     <row r="8" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5538,25 +5727,25 @@
         <v>0.00010416666555101983</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>503</v>
+        <v>520</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>504</v>
+        <v>521</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>505</v>
+        <v>522</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>506</v>
+        <v>523</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>507</v>
+        <v>524</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>508</v>
+        <v>525</v>
       </c>
     </row>
     <row r="9" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5574,30 +5763,30 @@
         <v>0.00028935185036971234</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>509</v>
+        <v>526</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>510</v>
+        <v>527</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>511</v>
+        <v>528</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>512</v>
+        <v>529</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>513</v>
+        <v>530</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>514</v>
+        <v>531</v>
       </c>
     </row>
     <row r="10" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>515</v>
+        <v>532</v>
       </c>
       <c r="B10" s="11">
         <v>46269.77627314815</v>
@@ -5613,27 +5802,27 @@
         <v>115</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>516</v>
+        <v>533</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>517</v>
+        <v>534</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>518</v>
+        <v>535</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>520</v>
+        <v>537</v>
       </c>
     </row>
     <row r="11" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
       <c r="B11" s="11">
         <v>46269.78513888889</v>
@@ -5646,30 +5835,30 @@
         <v>0.0005555555544560775</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>522</v>
+        <v>539</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>523</v>
+        <v>540</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>524</v>
+        <v>541</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>525</v>
+        <v>542</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>526</v>
+        <v>543</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>514</v>
+        <v>531</v>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>527</v>
+        <v>544</v>
       </c>
       <c r="B12" s="11">
         <v>46269.784733796296</v>
@@ -5682,30 +5871,30 @@
         <v>0.0009606481471564621</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>528</v>
+        <v>545</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>529</v>
+        <v>546</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>530</v>
+        <v>547</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>531</v>
+        <v>548</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>532</v>
+        <v>549</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>533</v>
+        <v>550</v>
       </c>
     </row>
     <row r="13" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>534</v>
+        <v>551</v>
       </c>
       <c r="B13" s="11">
         <v>46269.78622685185</v>
@@ -5721,16 +5910,16 @@
         <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>535</v>
+        <v>552</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>536</v>
+        <v>553</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>537</v>
+        <v>554</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>538</v>
+        <v>555</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>31</v>
@@ -5754,19 +5943,19 @@
         <v>0.0065393518525525</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>540</v>
+        <v>557</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -5786,25 +5975,25 @@
         <v>0.00020833333474001847</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>541</v>
+        <v>558</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>542</v>
+        <v>559</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>543</v>
+        <v>560</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>544</v>
+        <v>561</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>545</v>
+        <v>562</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>546</v>
+        <v>563</v>
       </c>
     </row>
     <row r="16" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5822,25 +6011,25 @@
         <v>0.0016666666670062114</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>547</v>
+        <v>564</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>549</v>
+        <v>566</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>551</v>
+        <v>568</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5861,16 +6050,16 @@
         <v>115</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>553</v>
+        <v>570</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>555</v>
+        <v>572</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>556</v>
+        <v>573</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>31</v>
@@ -5894,19 +6083,19 @@
         <v>0.01622685185066075</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>558</v>
+        <v>575</v>
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -5926,25 +6115,25 @@
         <v>0.0001851851848186925</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>559</v>
+        <v>576</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>560</v>
+        <v>577</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>561</v>
+        <v>578</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>562</v>
+        <v>579</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>563</v>
+        <v>580</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>564</v>
+        <v>581</v>
       </c>
     </row>
     <row r="20" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5962,25 +6151,25 @@
         <v>0.0015509259246755391</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>565</v>
+        <v>582</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>566</v>
+        <v>583</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>567</v>
+        <v>584</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>569</v>
+        <v>586</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
     </row>
     <row r="21" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5998,30 +6187,30 @@
         <v>0.001701388890069211</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>572</v>
+        <v>589</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>574</v>
+        <v>591</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>575</v>
+        <v>592</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>577</v>
+        <v>594</v>
       </c>
       <c r="B22" s="11">
         <v>46269.82821759259</v>
@@ -6034,30 +6223,30 @@
         <v>0.0010532407395658083</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>579</v>
+        <v>596</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>580</v>
+        <v>597</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>581</v>
+        <v>598</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>583</v>
+        <v>600</v>
       </c>
     </row>
     <row r="23" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>584</v>
+        <v>601</v>
       </c>
       <c r="B23" s="11">
         <v>46269.82745370371</v>
@@ -6070,30 +6259,30 @@
         <v>0.0033101851840910967</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>585</v>
+        <v>602</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>586</v>
+        <v>603</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>588</v>
+        <v>605</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>589</v>
+        <v>606</v>
       </c>
     </row>
     <row r="24" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>590</v>
+        <v>607</v>
       </c>
       <c r="B24" s="11">
         <v>46269.83311342592</v>
@@ -6109,16 +6298,16 @@
         <v>115</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>591</v>
+        <v>608</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>593</v>
+        <v>610</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>594</v>
+        <v>611</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>31</v>
@@ -6142,19 +6331,19 @@
         <v>0.03422453703751671</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>596</v>
+        <v>613</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
@@ -6174,25 +6363,25 @@
         <v>0.0005439814813144039</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>597</v>
+        <v>614</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>598</v>
+        <v>615</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>600</v>
+        <v>617</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>601</v>
+        <v>618</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>602</v>
+        <v>619</v>
       </c>
     </row>
     <row r="27" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6210,25 +6399,25 @@
         <v>0.0009375000008731149</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>603</v>
+        <v>620</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>604</v>
+        <v>621</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>605</v>
+        <v>622</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>606</v>
+        <v>623</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>607</v>
+        <v>624</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>608</v>
+        <v>625</v>
       </c>
     </row>
     <row r="28" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6246,25 +6435,25 @@
         <v>0.001574074074596865</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>609</v>
+        <v>626</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>610</v>
+        <v>627</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>611</v>
+        <v>628</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>612</v>
+        <v>629</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>613</v>
+        <v>630</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>614</v>
+        <v>631</v>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6317,19 +6506,19 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>616</v>
+        <v>633</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
@@ -6349,25 +6538,25 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>617</v>
+        <v>634</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>618</v>
+        <v>635</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>619</v>
+        <v>636</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>620</v>
+        <v>637</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>621</v>
+        <v>638</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>622</v>
+        <v>639</v>
       </c>
     </row>
     <row r="32" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6385,25 +6574,25 @@
         <v>0.0016319444439432118</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>623</v>
+        <v>640</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>624</v>
+        <v>641</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>625</v>
+        <v>642</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>626</v>
+        <v>643</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>627</v>
+        <v>644</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>628</v>
+        <v>645</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6421,19 +6610,19 @@
         <v>0.009606481482478557</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>629</v>
+        <v>646</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>629</v>
+        <v>646</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>629</v>
+        <v>646</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>629</v>
+        <v>646</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>630</v>
+        <v>647</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -6453,25 +6642,25 @@
         <v>0.0014351851859828457</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>631</v>
+        <v>648</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>632</v>
+        <v>649</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>633</v>
+        <v>650</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>634</v>
+        <v>651</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>635</v>
+        <v>652</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>636</v>
+        <v>653</v>
       </c>
     </row>
     <row r="35" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6489,25 +6678,25 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>637</v>
+        <v>654</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>638</v>
+        <v>655</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>639</v>
+        <v>656</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>640</v>
+        <v>657</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>641</v>
+        <v>658</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>642</v>
+        <v>659</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6518,26 +6707,26 @@
         <v>46270.46361111111</v>
       </c>
       <c r="C36" s="8">
-        <v>46270.47930555556</v>
+        <v>46270.47898148149</v>
       </c>
       <c r="D36" s="9">
         <f>C36-B36</f>
-        <v>0.015694444446126</v>
+        <v>0.015370370369055308</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>644</v>
+        <v>661</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
@@ -6557,30 +6746,30 @@
         <v>0.0014583333322661929</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>645</v>
+        <v>662</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>646</v>
+        <v>663</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>647</v>
+        <v>664</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>648</v>
+        <v>665</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>649</v>
+        <v>666</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>650</v>
+        <v>667</v>
       </c>
     </row>
     <row r="38" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>651</v>
+        <v>668</v>
       </c>
       <c r="B38" s="11">
         <v>46270.46697916667</v>
@@ -6593,30 +6782,30 @@
         <v>0.0029629629643750377</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>652</v>
+        <v>669</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>653</v>
+        <v>670</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>654</v>
+        <v>671</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>655</v>
+        <v>672</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>656</v>
+        <v>673</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>657</v>
+        <v>674</v>
       </c>
     </row>
     <row r="39" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>658</v>
+        <v>675</v>
       </c>
       <c r="B39" s="11">
         <v>46270.46810185185</v>
@@ -6629,30 +6818,30 @@
         <v>0.0006712962967867497</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>659</v>
+        <v>676</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>660</v>
+        <v>677</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>661</v>
+        <v>678</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>662</v>
+        <v>679</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>663</v>
+        <v>680</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>664</v>
+        <v>681</v>
       </c>
     </row>
     <row r="40" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>665</v>
+        <v>682</v>
       </c>
       <c r="B40" s="11">
         <v>46270.466782407406</v>
@@ -6665,30 +6854,30 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>666</v>
+        <v>683</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>667</v>
+        <v>684</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>668</v>
+        <v>685</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>669</v>
+        <v>686</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>670</v>
+        <v>687</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>657</v>
+        <v>674</v>
       </c>
     </row>
     <row r="41" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>671</v>
+        <v>688</v>
       </c>
       <c r="B41" s="11">
         <v>46270.471192129626</v>
@@ -6704,16 +6893,16 @@
         <v>115</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>672</v>
+        <v>689</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>673</v>
+        <v>690</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>674</v>
+        <v>691</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>675</v>
+        <v>692</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>31</v>
@@ -6724,38 +6913,142 @@
     </row>
     <row r="42" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>676</v>
+        <v>693</v>
       </c>
       <c r="B42" s="11">
         <v>46270.47395833333</v>
       </c>
       <c r="C42" s="11">
-        <v>46270.47930555556</v>
+        <v>46270.47898148149</v>
       </c>
       <c r="D42" s="12">
         <f>C42-B42</f>
-        <v>0.005347222220734693</v>
+        <v>0.005023148147301981</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>645</v>
+        <v>662</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>677</v>
+        <v>694</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>678</v>
+        <v>695</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>679</v>
+        <v>696</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>680</v>
+        <v>697</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>681</v>
+        <v>698</v>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="B43" s="8">
+        <v>46270.61494212963</v>
+      </c>
+      <c r="C43" s="8">
+        <v>46270.61938657408</v>
+      </c>
+      <c r="D43" s="9">
+        <f>C43-B43</f>
+        <v>0.004444444442924578</v>
+      </c>
+      <c r="E43" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="F43" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="G43" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="H43" s="7" t="s">
+        <v>699</v>
+      </c>
+      <c r="I43" s="7" t="s">
+        <v>700</v>
+      </c>
+      <c r="J43" s="7"/>
+      <c r="K43" s="7"/>
+    </row>
+    <row r="44" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" s="10" t="s">
+        <v>359</v>
+      </c>
+      <c r="B44" s="11">
+        <v>46270.61576388888</v>
+      </c>
+      <c r="C44" s="11">
+        <v>46270.616736111115</v>
+      </c>
+      <c r="D44" s="12">
+        <f>C44-B44</f>
+        <v>0.0009722222239361145</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>701</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>702</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>703</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>704</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>705</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="B45" s="11">
+        <v>46270.618680555555</v>
+      </c>
+      <c r="C45" s="11">
+        <v>46270.61938657408</v>
+      </c>
+      <c r="D45" s="12">
+        <f>C45-B45</f>
+        <v>0.0007060185198497493</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>708</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>709</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>710</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>711</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>120</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add image handling capabilities to the spreadsheet
- Enhance the Clipboard interface to include image sizes for copied cells.
- Implement copyRange function to capture image sizes when copying cells with images.
- Introduce pasteSizes function to handle the positioning of pasted images.
- Create ImageTransformBox component for resizing images within cells.
- Add tests for clipboard image handling and image transformation functionalities.
- Implement imageFromClipboard function to determine if the clipboard contains an image.
- Develop imageTransform functions to manage resizing behavior and aspect ratios.
</commit_message>
<xml_diff>
--- a/Cowork changes 4 Sep 2026.xlsx
+++ b/Cowork changes 4 Sep 2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="948" uniqueCount="712">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="988" uniqueCount="747">
   <si>
     <t>Cowork — changes, 4 September 2026</t>
   </si>
@@ -1254,6 +1254,111 @@
   </si>
   <si>
     <t>components/features/spreadsheet/{useSpreadsheet,CellVisual}.tsx; components/ui/DriveImage.tsx</t>
+  </si>
+  <si>
+    <t>11c</t>
+  </si>
+  <si>
+    <t>Sheets ▸ double-click a cell holding a picture</t>
+  </si>
+  <si>
+    <t>A resize box on the picture, instead of the formula editor</t>
+  </si>
+  <si>
+    <t>Double-clicking a picture opened the cell editor, which showed the raw =IMAGE("https://lh3.googleusercontent.com/d/124CC…=w1600") — a line of machine address where a picture had been. It is what the cell holds, but not what anybody double-clicked a picture to get, and there was no way at all to resize the thing on screen.</t>
+  </si>
+  <si>
+    <t>A box round the picture with eight handles. A corner keeps its proportions, a side stretches one way, the cell follows the box, and the figure under the hand says what size it is becoming. Escape or a click elsewhere puts it away. Nothing is capped — this is after the import, which is the distinction asked for. The formula bar still shows the address and F2 still opens the editor, so nothing was taken away; it is only no longer what the gesture means.</t>
+  </si>
+  <si>
+    <t>The arithmetic is a pure module with 15 tests — which handle keeps the ratio, why a north or west drag means BIGGER (the cell’s top-left is pinned to the grid and cannot move), and why a corner follows whichever axis moved further as a FRACTION of the starting size rather than in raw pixels, or the wide axis wins every time on a wide picture and the box ignores vertical movement. The ratio is the PICTURE’s, not the cell’s, so a cell somebody already squashed snaps back to the true shape on the first corner drag instead of preserving the distortion for ever.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/{ImageTransformBox,SpreadsheetGrid,useSpreadsheet}.tsx; lib/spreadsheet/imageTransform.ts; lib/help/knowledge.ts</t>
+  </si>
+  <si>
+    <t>11d</t>
+  </si>
+  <si>
+    <t>Sheets ▸ the picture resize box</t>
+  </si>
+  <si>
+    <t>Two defects the browser found that the code did not</t>
+  </si>
+  <si>
+    <t>First: nothing happened when a handle was dragged. The grid’s drag-to-fill handle sits at the selection’s bottom-right and so does the box’s own SE handle — the same pixel meaning two things — and the fill handle sits at z-20 against the box’s z-6, so it took every pointer. The drag became a selection and the sheet auto-scrolled to AF1:AH6. Second, once that was fixed: a drag committed the new HEIGHT and silently kept the old width.</t>
+  </si>
+  <si>
+    <t>The fill handle stands down while the box is open — the box owns the cell — and the box sits above the selection chrome at z-21. The width and height are now committed as ONE command, `resizeCell`, which is also one undo for one drag.</t>
+  </si>
+  <si>
+    <t>The second was the interesting one. `resizeCol` and `resizeRow` each build their next worksheet from the SAME render’s `worksheet`, so calling them one after the other in a single handler means the second’s result never contains the first’s change and quietly discards it. Nothing about the code looks wrong; a drag to 250 × 124 simply produced 100 × 124 on screen. The same trap was already avoided in `insertImageCell`, where the two sizes were composed into one worksheet — this makes that composition a method rather than a thing each caller has to remember.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/{SpreadsheetGrid,useSpreadsheet,ImageTransformBox}.tsx</t>
+  </si>
+  <si>
+    <t>11e</t>
+  </si>
+  <si>
+    <t>Sheets ▸ pasting into a cell</t>
+  </si>
+  <si>
+    <t>Paste a picture from the clipboard, and copy one between cells</t>
+  </si>
+  <si>
+    <t>Neither worked. Pasting a screenshot did nothing at all, because `controller.paste()` reads the clipboard through `navigator.clipboard.readText()` — which can only ever see text, never bytes. And copying a picture from one cell to another carried the =IMAGE formula but not the cell’s size, so it arrived in a default 100 × 24 cell: the same picture, cropped.</t>
+  </si>
+  <si>
+    <t>A picture on the system clipboard opens the SAME editor Insert ▸ Image opens — it has not been cropped or sized yet and still has to be uploaded. A picture copied from one CELL to another opens nothing: it arrives at the size it already had, crop and rotation included, because that was settled once at import and a copy is not a re-import. Cut behaves the same; the picture is moving, not being retyped.</t>
+  </si>
+  <si>
+    <t>The interesting decision is which paste is which. A range copied out of Excel or Google Sheets carries tab-separated text, HTML AND a bitmap of the cells, so “does the clipboard hold an image?” is true for a screenshot and for somebody’s numbers alike — answering yes to both would hijack every ordinary paste and offer to crop a picture of a spreadsheet. The rule is therefore: a picture only when there is no TEXT to paste instead. Ten tests cover it. The size travels in its own field rather than alongside the styles, and only for cells that actually held a picture: a row height and a column width belong to the row and the column, so carrying them for every copied cell would mean an ordinary paste of text silently resized whatever it landed on.</t>
+  </si>
+  <si>
+    <t>lib/spreadsheet/{clipboard,clipboardImage}.ts (+ 20 tests); components/features/spreadsheet/{SpreadsheetGrid,useSpreadsheet}.tsx; lib/help/knowledge.ts</t>
+  </si>
+  <si>
+    <t>11f</t>
+  </si>
+  <si>
+    <t>Sheets ▸ pasting a picture between cells</t>
+  </si>
+  <si>
+    <t>The pasted cell kept its size and lost its value</t>
+  </si>
+  <si>
+    <t>Seen in a browser, not in the code: the destination cell drew the picture and took the right size, and its formula bar was EMPTY. The size was applied in a second structural command after the values — and `applyStructural` REPLACES the worksheet with one computed from the render it was called in, while `applyEdits` applies its changes functionally to whatever is current. So the size command, built from the pre-paste worksheet, threw the pasted values away; and because it passes `rebuild: false` the formula engine kept them, which is why the cell went on drawing a picture it no longer contained.</t>
+  </si>
+  <si>
+    <t>The sizes are applied BEFORE the values. Verified: pasting a 252 × 124 picture from A1 into D7 now gives D7 both the formula and the size, with every other column still at its default 100.</t>
+  </si>
+  <si>
+    <t>Third time this exact trap has appeared today — `insertImageCell` avoided it by accident of ordering, `resizeCell` was created to escape it, and here it bit. The rule is worth stating plainly: in this hook a structural apply must never follow an edits apply in the same handler. Pinned by a test that compares the two positions rather than describing the rule in prose.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/useSpreadsheet.ts</t>
+  </si>
+  <si>
+    <t>11g</t>
+  </si>
+  <si>
+    <t>Sheets ▸ Ctrl+V</t>
+  </si>
+  <si>
+    <t>Pasting a picture from the clipboard actually works now</t>
+  </si>
+  <si>
+    <t>11e added the handler and it could never run. The grid claims Ctrl+V on keydown with `preventDefault()`, and a prevented Ctrl+V means the browser never generates a `paste` event at all — and that event is the only thing that carries clipboard BYTES. So the picture handler was correct and unreachable. Reported by the owner as “still isn’t working”.</t>
+  </si>
+  <si>
+    <t>Ctrl+V no longer prevents the default; it only stops the shortcut reaching the app shell. The paste event now does the whole job — a picture opens the import editor, and text is placed from the text the EVENT carries rather than by reading the clipboard again. Copy and cut still claim their keys, because they act on the selection and want no payload back.</t>
+  </si>
+  <si>
+    <t>My own verification of 11e is what hid this. I dispatched a synthetic `ClipboardEvent` straight at the grid, which reaches the handler without going near the keyboard — so it proved the handler worked and said nothing about whether anything could ever call it. The fix is verified the other way round: with the grid focused, Ctrl+V now reports defaultPrevented FALSE while Ctrl+C still reports true. Reading the clipboard from the event is better anyway: `navigator.clipboard.readText()` needs a permission the event does not, and can never see bytes.</t>
+  </si>
+  <si>
+    <t>components/features/spreadsheet/{SpreadsheetGrid,useSpreadsheet}.tsx (+ 4 regression tests)</t>
   </si>
   <si>
     <t>What is open</t>
@@ -2844,7 +2949,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K64"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -4749,11 +4854,11 @@
         <v>46270.52013888889</v>
       </c>
       <c r="C57" s="8">
-        <v>46270.62466435185</v>
+        <v>46270.69208333333</v>
       </c>
       <c r="D57" s="9">
         <f>C57-B57</f>
-        <v>0.10452546296296296</v>
+        <v>0.17194444444444446</v>
       </c>
       <c r="E57" s="7" t="s">
         <v>367</v>
@@ -4919,11 +5024,11 @@
         <v>46270.55902777778</v>
       </c>
       <c r="C62" s="8">
-        <v>46270.62466435185</v>
+        <v>46270.69208333333</v>
       </c>
       <c r="D62" s="9">
         <f>C62-B62</f>
-        <v>0.06563657407407407</v>
+        <v>0.13305555555555557</v>
       </c>
       <c r="E62" s="7" t="s">
         <v>397</v>
@@ -4945,11 +5050,11 @@
         <v>46270.55902777778</v>
       </c>
       <c r="C63" s="11">
-        <v>46270.62466435185</v>
+        <v>46270.69208333333</v>
       </c>
       <c r="D63" s="12">
         <f>C63-B63</f>
-        <v>0.06563657407407407</v>
+        <v>0.13305555555555557</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>400</v>
@@ -4981,11 +5086,11 @@
         <v>46270.61458333333</v>
       </c>
       <c r="C64" s="11">
-        <v>46270.62466435185</v>
+        <v>46270.62361111111</v>
       </c>
       <c r="D64" s="12">
         <f>C64-B64</f>
-        <v>0.010081018518518519</v>
+        <v>0.009027777777777777</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>407</v>
@@ -5009,8 +5114,188 @@
         <v>412</v>
       </c>
     </row>
+    <row r="65" ht="188" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="B65" s="11">
+        <v>46270.62430555555</v>
+      </c>
+      <c r="C65" s="11">
+        <v>46270.69208333333</v>
+      </c>
+      <c r="D65" s="12">
+        <f>C65-B65</f>
+        <v>0.06777777777777778</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>415</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K65" s="2" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="66" ht="188" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="B66" s="11">
+        <v>46270.62847222222</v>
+      </c>
+      <c r="C66" s="11">
+        <v>46270.638194444444</v>
+      </c>
+      <c r="D66" s="12">
+        <f>C66-B66</f>
+        <v>0.009722222222222222</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>421</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="I66" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K66" s="2" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="67" ht="244" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="B67" s="11">
+        <v>46270.63888888889</v>
+      </c>
+      <c r="C67" s="11">
+        <v>46270.69208333333</v>
+      </c>
+      <c r="D67" s="12">
+        <f>C67-B67</f>
+        <v>0.05319444444444445</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K67" s="2" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="68" ht="216" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="B68" s="11">
+        <v>46270.65277777778</v>
+      </c>
+      <c r="C68" s="11">
+        <v>46270.6625</v>
+      </c>
+      <c r="D68" s="12">
+        <f>C68-B68</f>
+        <v>0.009722222222222222</v>
+      </c>
+      <c r="E68" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="F68" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>437</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K68" s="2" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="69" ht="174" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A69" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="B69" s="11">
+        <v>46270.66666666667</v>
+      </c>
+      <c r="C69" s="11">
+        <v>46270.69208333333</v>
+      </c>
+      <c r="D69" s="12">
+        <f>C69-B69</f>
+        <v>0.025416666666666667</v>
+      </c>
+      <c r="E69" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="F69" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>444</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>445</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K69" s="2" t="s">
+        <v>447</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K64"/>
+  <autoFilter ref="A1:K69"/>
   <mergeCells count="13">
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="E3:H3"/>
@@ -5046,13 +5331,13 @@
         <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>413</v>
+        <v>448</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>414</v>
+        <v>449</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>415</v>
+        <v>450</v>
       </c>
     </row>
     <row r="2" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5060,27 +5345,27 @@
         <v>137</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>416</v>
+        <v>451</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>417</v>
+        <v>452</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>418</v>
+        <v>453</v>
       </c>
     </row>
     <row r="3" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>419</v>
+        <v>454</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>420</v>
+        <v>455</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>421</v>
+        <v>456</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>422</v>
+        <v>457</v>
       </c>
     </row>
     <row r="4" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5088,13 +5373,13 @@
         <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>423</v>
+        <v>458</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>424</v>
+        <v>459</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>425</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5102,13 +5387,13 @@
         <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>426</v>
+        <v>461</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>427</v>
+        <v>462</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>428</v>
+        <v>463</v>
       </c>
     </row>
     <row r="6" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5116,13 +5401,13 @@
         <v>108</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>429</v>
+        <v>464</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>431</v>
+        <v>466</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5130,13 +5415,13 @@
         <v>176</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>433</v>
+        <v>468</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>434</v>
+        <v>469</v>
       </c>
     </row>
     <row r="8" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5144,27 +5429,27 @@
         <v>176</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>435</v>
+        <v>470</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>436</v>
+        <v>471</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>437</v>
+        <v>472</v>
       </c>
     </row>
     <row r="9" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>438</v>
+        <v>473</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>439</v>
+        <v>474</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>441</v>
+        <v>476</v>
       </c>
     </row>
     <row r="10" ht="80" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5172,13 +5457,13 @@
         <v>251</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>442</v>
+        <v>477</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>444</v>
+        <v>479</v>
       </c>
     </row>
     <row r="11" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5186,13 +5471,13 @@
         <v>199</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>446</v>
+        <v>481</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>447</v>
+        <v>482</v>
       </c>
     </row>
     <row r="12" ht="66" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5200,13 +5485,13 @@
         <v>199</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>448</v>
+        <v>483</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
     </row>
     <row r="13" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -5214,27 +5499,27 @@
         <v>199</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>451</v>
+        <v>486</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>452</v>
+        <v>487</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>453</v>
+        <v>488</v>
       </c>
     </row>
     <row r="14" ht="52" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>454</v>
+        <v>489</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>455</v>
+        <v>490</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>456</v>
+        <v>491</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>457</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -5257,7 +5542,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>458</v>
+        <v>493</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -5270,179 +5555,179 @@
         <v>40</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>459</v>
+        <v>494</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>460</v>
+        <v>495</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>461</v>
+        <v>496</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>462</v>
+        <v>497</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>463</v>
+        <v>498</v>
       </c>
     </row>
     <row r="3" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>464</v>
+        <v>499</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>465</v>
+        <v>500</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>466</v>
+        <v>501</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>467</v>
+        <v>502</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="4" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>470</v>
+        <v>505</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>471</v>
+        <v>506</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>472</v>
+        <v>507</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>473</v>
+        <v>508</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>474</v>
+        <v>509</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>218</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>475</v>
+        <v>510</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>476</v>
+        <v>511</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>477</v>
+        <v>512</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>199</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>479</v>
+        <v>514</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>480</v>
+        <v>515</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>481</v>
+        <v>516</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="7" ht="50" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>206</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>483</v>
+        <v>518</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>484</v>
+        <v>519</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="8" ht="92" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>261</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>487</v>
+        <v>522</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>488</v>
+        <v>523</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>489</v>
+        <v>524</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>490</v>
+        <v>525</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>491</v>
+        <v>526</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>492</v>
+        <v>527</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>494</v>
+        <v>529</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
     <row r="10" ht="78" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>495</v>
+        <v>530</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>496</v>
+        <v>531</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>497</v>
+        <v>532</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>498</v>
+        <v>533</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>499</v>
+        <v>534</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -5567,7 +5852,7 @@
         <v>322</v>
       </c>
       <c r="I3" s="7" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
@@ -5590,22 +5875,22 @@
         <v>159</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>501</v>
+        <v>536</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>503</v>
+        <v>538</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>504</v>
+        <v>539</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>505</v>
+        <v>540</v>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5623,19 +5908,19 @@
         <v>0.017418981482478557</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="I5" s="7" t="s">
-        <v>507</v>
+        <v>542</v>
       </c>
       <c r="J5" s="7"/>
       <c r="K5" s="7"/>
@@ -5655,25 +5940,25 @@
         <v>0.0020370370366435964</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>508</v>
+        <v>543</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>510</v>
+        <v>545</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>511</v>
+        <v>546</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>512</v>
+        <v>547</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>513</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5691,25 +5976,25 @@
         <v>0.0026504629640839994</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>514</v>
+        <v>549</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>515</v>
+        <v>550</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>516</v>
+        <v>551</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>517</v>
+        <v>552</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>518</v>
+        <v>553</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>519</v>
+        <v>554</v>
       </c>
     </row>
     <row r="8" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5727,25 +6012,25 @@
         <v>0.00010416666555101983</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>520</v>
+        <v>555</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>521</v>
+        <v>556</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>522</v>
+        <v>557</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>523</v>
+        <v>558</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>524</v>
+        <v>559</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>525</v>
+        <v>560</v>
       </c>
     </row>
     <row r="9" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -5763,30 +6048,30 @@
         <v>0.00028935185036971234</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>526</v>
+        <v>561</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>527</v>
+        <v>562</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>528</v>
+        <v>563</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>529</v>
+        <v>564</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>530</v>
+        <v>565</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="10" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
       <c r="B10" s="11">
         <v>46269.77627314815</v>
@@ -5802,27 +6087,27 @@
         <v>115</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>533</v>
+        <v>568</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>534</v>
+        <v>569</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>535</v>
+        <v>570</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>536</v>
+        <v>571</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>537</v>
+        <v>572</v>
       </c>
     </row>
     <row r="11" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>538</v>
+        <v>573</v>
       </c>
       <c r="B11" s="11">
         <v>46269.78513888889</v>
@@ -5835,30 +6120,30 @@
         <v>0.0005555555544560775</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>539</v>
+        <v>574</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>540</v>
+        <v>575</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>541</v>
+        <v>576</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>544</v>
+        <v>579</v>
       </c>
       <c r="B12" s="11">
         <v>46269.784733796296</v>
@@ -5871,30 +6156,30 @@
         <v>0.0009606481471564621</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>545</v>
+        <v>580</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>546</v>
+        <v>581</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>547</v>
+        <v>582</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>548</v>
+        <v>583</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>549</v>
+        <v>584</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>550</v>
+        <v>585</v>
       </c>
     </row>
     <row r="13" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>551</v>
+        <v>586</v>
       </c>
       <c r="B13" s="11">
         <v>46269.78622685185</v>
@@ -5910,16 +6195,16 @@
         <v>115</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>552</v>
+        <v>587</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>553</v>
+        <v>588</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>554</v>
+        <v>589</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>555</v>
+        <v>590</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>31</v>
@@ -5943,19 +6228,19 @@
         <v>0.0065393518525525</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>557</v>
+        <v>592</v>
       </c>
       <c r="J14" s="7"/>
       <c r="K14" s="7"/>
@@ -5975,25 +6260,25 @@
         <v>0.00020833333474001847</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>558</v>
+        <v>593</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>559</v>
+        <v>594</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>560</v>
+        <v>595</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>561</v>
+        <v>596</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>562</v>
+        <v>597</v>
       </c>
       <c r="J15" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>563</v>
+        <v>598</v>
       </c>
     </row>
     <row r="16" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6011,25 +6296,25 @@
         <v>0.0016666666670062114</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>564</v>
+        <v>599</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>565</v>
+        <v>600</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>566</v>
+        <v>601</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>567</v>
+        <v>602</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>568</v>
+        <v>603</v>
       </c>
       <c r="J16" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>569</v>
+        <v>604</v>
       </c>
     </row>
     <row r="17" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6050,16 +6335,16 @@
         <v>115</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>570</v>
+        <v>605</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>571</v>
+        <v>606</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>572</v>
+        <v>607</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>573</v>
+        <v>608</v>
       </c>
       <c r="J17" s="2" t="s">
         <v>31</v>
@@ -6083,19 +6368,19 @@
         <v>0.01622685185066075</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>574</v>
+        <v>609</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>575</v>
+        <v>610</v>
       </c>
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
@@ -6115,25 +6400,25 @@
         <v>0.0001851851848186925</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>576</v>
+        <v>611</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>577</v>
+        <v>612</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>578</v>
+        <v>613</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>579</v>
+        <v>614</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>580</v>
+        <v>615</v>
       </c>
       <c r="J19" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K19" s="2" t="s">
-        <v>581</v>
+        <v>616</v>
       </c>
     </row>
     <row r="20" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6151,25 +6436,25 @@
         <v>0.0015509259246755391</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>582</v>
+        <v>617</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>583</v>
+        <v>618</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>584</v>
+        <v>619</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>585</v>
+        <v>620</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>586</v>
+        <v>621</v>
       </c>
       <c r="J20" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K20" s="2" t="s">
-        <v>587</v>
+        <v>622</v>
       </c>
     </row>
     <row r="21" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6187,30 +6472,30 @@
         <v>0.001701388890069211</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>588</v>
+        <v>623</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>589</v>
+        <v>624</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>590</v>
+        <v>625</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>591</v>
+        <v>626</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>592</v>
+        <v>627</v>
       </c>
       <c r="J21" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K21" s="2" t="s">
-        <v>593</v>
+        <v>628</v>
       </c>
     </row>
     <row r="22" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
-        <v>594</v>
+        <v>629</v>
       </c>
       <c r="B22" s="11">
         <v>46269.82821759259</v>
@@ -6223,30 +6508,30 @@
         <v>0.0010532407395658083</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>595</v>
+        <v>630</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>596</v>
+        <v>631</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>597</v>
+        <v>632</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>598</v>
+        <v>633</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>599</v>
+        <v>634</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K22" s="2" t="s">
-        <v>600</v>
+        <v>635</v>
       </c>
     </row>
     <row r="23" ht="118" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="10" t="s">
-        <v>601</v>
+        <v>636</v>
       </c>
       <c r="B23" s="11">
         <v>46269.82745370371</v>
@@ -6259,30 +6544,30 @@
         <v>0.0033101851840910967</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>595</v>
+        <v>630</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>602</v>
+        <v>637</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>603</v>
+        <v>638</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>604</v>
+        <v>639</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>605</v>
+        <v>640</v>
       </c>
       <c r="J23" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K23" s="2" t="s">
-        <v>606</v>
+        <v>641</v>
       </c>
     </row>
     <row r="24" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="10" t="s">
-        <v>607</v>
+        <v>642</v>
       </c>
       <c r="B24" s="11">
         <v>46269.83311342592</v>
@@ -6298,16 +6583,16 @@
         <v>115</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>608</v>
+        <v>643</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>609</v>
+        <v>644</v>
       </c>
       <c r="H24" s="2" t="s">
-        <v>610</v>
+        <v>645</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>611</v>
+        <v>646</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>31</v>
@@ -6331,19 +6616,19 @@
         <v>0.03422453703751671</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>612</v>
+        <v>647</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>613</v>
+        <v>648</v>
       </c>
       <c r="J25" s="7"/>
       <c r="K25" s="7"/>
@@ -6363,25 +6648,25 @@
         <v>0.0005439814813144039</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>614</v>
+        <v>649</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>615</v>
+        <v>650</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>616</v>
+        <v>651</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>617</v>
+        <v>652</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>618</v>
+        <v>653</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K26" s="2" t="s">
-        <v>619</v>
+        <v>654</v>
       </c>
     </row>
     <row r="27" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6399,25 +6684,25 @@
         <v>0.0009375000008731149</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>620</v>
+        <v>655</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>621</v>
+        <v>656</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>622</v>
+        <v>657</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>623</v>
+        <v>658</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>624</v>
+        <v>659</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K27" s="2" t="s">
-        <v>625</v>
+        <v>660</v>
       </c>
     </row>
     <row r="28" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6435,25 +6720,25 @@
         <v>0.001574074074596865</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>626</v>
+        <v>661</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>627</v>
+        <v>662</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>628</v>
+        <v>663</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>629</v>
+        <v>664</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>630</v>
+        <v>665</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K28" s="2" t="s">
-        <v>631</v>
+        <v>666</v>
       </c>
     </row>
     <row r="29" ht="26" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6506,19 +6791,19 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>632</v>
+        <v>667</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>632</v>
+        <v>667</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>632</v>
+        <v>667</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>632</v>
+        <v>667</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>633</v>
+        <v>668</v>
       </c>
       <c r="J30" s="7"/>
       <c r="K30" s="7"/>
@@ -6538,25 +6823,25 @@
         <v>0.002858796295186039</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>634</v>
+        <v>669</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>635</v>
+        <v>670</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>636</v>
+        <v>671</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>637</v>
+        <v>672</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>638</v>
+        <v>673</v>
       </c>
       <c r="J31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="2" t="s">
-        <v>639</v>
+        <v>674</v>
       </c>
     </row>
     <row r="32" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6574,25 +6859,25 @@
         <v>0.0016319444439432118</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>640</v>
+        <v>675</v>
       </c>
       <c r="F32" s="2" t="s">
-        <v>641</v>
+        <v>676</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>642</v>
+        <v>677</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>643</v>
+        <v>678</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>644</v>
+        <v>679</v>
       </c>
       <c r="J32" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>645</v>
+        <v>680</v>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6610,19 +6895,19 @@
         <v>0.009606481482478557</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>646</v>
+        <v>681</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>647</v>
+        <v>682</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -6642,25 +6927,25 @@
         <v>0.0014351851859828457</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>648</v>
+        <v>683</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>649</v>
+        <v>684</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>650</v>
+        <v>685</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>651</v>
+        <v>686</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>652</v>
+        <v>687</v>
       </c>
       <c r="J34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>653</v>
+        <v>688</v>
       </c>
     </row>
     <row r="35" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6678,25 +6963,25 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>654</v>
+        <v>689</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>655</v>
+        <v>690</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>656</v>
+        <v>691</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>657</v>
+        <v>692</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>658</v>
+        <v>693</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>659</v>
+        <v>694</v>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6714,19 +6999,19 @@
         <v>0.015370370369055308</v>
       </c>
       <c r="E36" s="7" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
       <c r="H36" s="7" t="s">
-        <v>660</v>
+        <v>695</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>661</v>
+        <v>696</v>
       </c>
       <c r="J36" s="7"/>
       <c r="K36" s="7"/>
@@ -6746,30 +7031,30 @@
         <v>0.0014583333322661929</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>662</v>
+        <v>697</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>663</v>
+        <v>698</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>664</v>
+        <v>699</v>
       </c>
       <c r="H37" s="2" t="s">
-        <v>665</v>
+        <v>700</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>666</v>
+        <v>701</v>
       </c>
       <c r="J37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>667</v>
+        <v>702</v>
       </c>
     </row>
     <row r="38" ht="104" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" s="10" t="s">
-        <v>668</v>
+        <v>703</v>
       </c>
       <c r="B38" s="11">
         <v>46270.46697916667</v>
@@ -6782,30 +7067,30 @@
         <v>0.0029629629643750377</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>669</v>
+        <v>704</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>670</v>
+        <v>705</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>671</v>
+        <v>706</v>
       </c>
       <c r="H38" s="2" t="s">
-        <v>672</v>
+        <v>707</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>673</v>
+        <v>708</v>
       </c>
       <c r="J38" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>674</v>
+        <v>709</v>
       </c>
     </row>
     <row r="39" ht="76" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" s="10" t="s">
-        <v>675</v>
+        <v>710</v>
       </c>
       <c r="B39" s="11">
         <v>46270.46810185185</v>
@@ -6818,30 +7103,30 @@
         <v>0.0006712962967867497</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>676</v>
+        <v>711</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>677</v>
+        <v>712</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>678</v>
+        <v>713</v>
       </c>
       <c r="H39" s="2" t="s">
-        <v>679</v>
+        <v>714</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>680</v>
+        <v>715</v>
       </c>
       <c r="J39" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>681</v>
+        <v>716</v>
       </c>
     </row>
     <row r="40" ht="90" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>682</v>
+        <v>717</v>
       </c>
       <c r="B40" s="11">
         <v>46270.466782407406</v>
@@ -6854,30 +7139,30 @@
         <v>0.0005092592582514044</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>683</v>
+        <v>718</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>684</v>
+        <v>719</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>685</v>
+        <v>720</v>
       </c>
       <c r="H40" s="2" t="s">
-        <v>686</v>
+        <v>721</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>687</v>
+        <v>722</v>
       </c>
       <c r="J40" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>674</v>
+        <v>709</v>
       </c>
     </row>
     <row r="41" ht="62" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>688</v>
+        <v>723</v>
       </c>
       <c r="B41" s="11">
         <v>46270.471192129626</v>
@@ -6893,16 +7178,16 @@
         <v>115</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>689</v>
+        <v>724</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>690</v>
+        <v>725</v>
       </c>
       <c r="H41" s="2" t="s">
-        <v>691</v>
+        <v>726</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>692</v>
+        <v>727</v>
       </c>
       <c r="J41" s="2" t="s">
         <v>31</v>
@@ -6913,7 +7198,7 @@
     </row>
     <row r="42" ht="132" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>693</v>
+        <v>728</v>
       </c>
       <c r="B42" s="11">
         <v>46270.47395833333</v>
@@ -6926,25 +7211,25 @@
         <v>0.005023148147301981</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>662</v>
+        <v>697</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>694</v>
+        <v>729</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>695</v>
+        <v>730</v>
       </c>
       <c r="H42" s="2" t="s">
-        <v>696</v>
+        <v>731</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>697</v>
+        <v>732</v>
       </c>
       <c r="J42" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>698</v>
+        <v>733</v>
       </c>
     </row>
     <row r="43" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -6962,19 +7247,19 @@
         <v>0.004444444442924578</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>699</v>
+        <v>734</v>
       </c>
       <c r="F43" s="7" t="s">
-        <v>699</v>
+        <v>734</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>699</v>
+        <v>734</v>
       </c>
       <c r="H43" s="7" t="s">
-        <v>699</v>
+        <v>734</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>700</v>
+        <v>735</v>
       </c>
       <c r="J43" s="7"/>
       <c r="K43" s="7"/>
@@ -6994,30 +7279,30 @@
         <v>0.0009722222239361145</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>701</v>
+        <v>736</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>702</v>
+        <v>737</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>703</v>
+        <v>738</v>
       </c>
       <c r="H44" s="2" t="s">
-        <v>704</v>
+        <v>739</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>705</v>
+        <v>740</v>
       </c>
       <c r="J44" s="2" t="s">
         <v>31</v>
       </c>
       <c r="K44" s="2" t="s">
-        <v>706</v>
+        <v>741</v>
       </c>
     </row>
     <row r="45" ht="48" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>707</v>
+        <v>742</v>
       </c>
       <c r="B45" s="11">
         <v>46270.618680555555</v>
@@ -7033,16 +7318,16 @@
         <v>115</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>708</v>
+        <v>743</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>709</v>
+        <v>744</v>
       </c>
       <c r="H45" s="2" t="s">
-        <v>710</v>
+        <v>745</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>711</v>
+        <v>746</v>
       </c>
       <c r="J45" s="2" t="s">
         <v>31</v>

</xml_diff>